<commit_message>
Plan FridayJumaat at Tokyo Camii and fix Shibuya Sky price
</commit_message>
<xml_diff>
--- a/Japan_Winter_Trip_Itinerary.xlsx
+++ b/Japan_Winter_Trip_Itinerary.xlsx
@@ -1744,7 +1744,11 @@
       </c>
       <c r="E34" s="25" t="n"/>
       <c r="F34" s="25" t="n"/>
-      <c r="G34" s="25" t="n"/>
+      <c r="G34" s="25" t="inlineStr">
+        <is>
+          <t>Gerak ke Tokyo Camii ~11:30: Ginza Line → Omotesando, tukar Chiyoda Line → Yoyogi-Uehara (~40min)</t>
+        </is>
+      </c>
       <c r="H34" s="25" t="n"/>
       <c r="I34" s="26" t="n"/>
       <c r="J34" s="26" t="n"/>
@@ -1762,21 +1766,25 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>11:47</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="D35" s="27" t="inlineStr">
         <is>
-          <t>Zohor (cadangan: Tokyo Camii, Yoyogi-Uehara)</t>
+          <t>SOLAT JUMAAT kat Tokyo Camii (lelaki sampai sebelum 12:15). Perempuan: ikut Jumaat di ruang wanita, atau Zohor biasa</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
         <is>
-          <t>Zohor 11:47</t>
+          <t>Jumaat ~13:00 (azan ~12:30)</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
-      <c r="G35" s="27" t="n"/>
+      <c r="G35" s="27" t="inlineStr">
+        <is>
+          <t>Khutbah dalam bahasa Jepun, Turki &amp; Inggeris</t>
+        </is>
+      </c>
       <c r="H35" s="27" t="n"/>
       <c r="I35" s="28" t="n"/>
       <c r="J35" s="28" t="n"/>
@@ -1794,12 +1802,12 @@
       </c>
       <c r="C36" s="25" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D36" s="25" t="inlineStr">
         <is>
-          <t>Lunch — halal dekat Tokyo Camii/Shin-Okubo</t>
+          <t>Lunch — halal kat Tokyo Camii (market bawah) / Shin-Okubo, LEPAS Jumaat</t>
         </is>
       </c>
       <c r="E36" s="25" t="n"/>
@@ -2290,14 +2298,14 @@
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>Explore lagi (Shibuya Sky — OPTIONAL, boleh skip)</t>
+          <t>Shibuya Sky — slot 14:30 (OPTIONAL, boleh skip)</t>
         </is>
       </c>
       <c r="E50" s="25" t="n"/>
       <c r="F50" s="25" t="n"/>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>Optional attraction</t>
+          <t>¥2,700 online (slot sebelum 15:00). Tiket buka 26 Dis 00:00. Keluar sebelum Maghrib ~16:45</t>
         </is>
       </c>
       <c r="H50" s="25" t="inlineStr">
@@ -2306,7 +2314,7 @@
         </is>
       </c>
       <c r="I50" s="26" t="n">
-        <v>2000</v>
+        <v>2700</v>
       </c>
       <c r="J50" s="26">
         <f>I50*'Budget Summary'!$B$2</f>

</xml_diff>

<commit_message>
Replace cloud restaurants and switch Fuji leg to a rental car
</commit_message>
<xml_diff>
--- a/Japan_Winter_Trip_Itinerary.xlsx
+++ b/Japan_Winter_Trip_Itinerary.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="22" min="1" max="1"/>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="C44" s="25" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="D44" s="25" t="inlineStr">
@@ -2123,89 +2123,106 @@
       </c>
       <c r="C45" s="25" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="D45" s="25" t="inlineStr">
         <is>
-          <t>Local transport Tokyo</t>
+          <t>Check-out manga cafe, bawa SEMUA bagasi ke Toyota Rent a Car Shinjuku</t>
         </is>
       </c>
       <c r="E45" s="25" t="n"/>
       <c r="F45" s="25" t="n"/>
-      <c r="G45" s="25" t="n"/>
-      <c r="H45" s="25" t="inlineStr">
+      <c r="G45" s="25" t="inlineStr">
+        <is>
+          <t>Beli kairo (heat pack) + air kat konbini untuk malam ni</t>
+        </is>
+      </c>
+      <c r="H45" s="25" t="n"/>
+      <c r="I45" s="26" t="n"/>
+      <c r="J45" s="26" t="n"/>
+    </row>
+    <row r="46" ht="27.75" customHeight="1" s="23">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D46" s="31" t="inlineStr">
+        <is>
+          <t>AMBIL KERETA — Toyota Noah/Voxy (kelas W2, 7-8 seat) + tayar salji + kad ETC</t>
+        </is>
+      </c>
+      <c r="E46" s="31" t="n"/>
+      <c r="F46" s="31" t="n"/>
+      <c r="G46" s="31" t="inlineStr">
+        <is>
+          <t>WAJIB: passport + lesen Malaysia + IDP (buku fizikal) untuk 3 pemandu. Sewa ~¥37-45k + tayar salji ¥3,300/24j + insurans ≈ ¥52k ÷ 6</t>
+        </is>
+      </c>
+      <c r="H46" s="31" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="I45" s="26" t="n">
-        <v>800</v>
-      </c>
-      <c r="J45" s="26">
-        <f>I45*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="27.75" customHeight="1" s="23">
-      <c r="A46" s="25" t="inlineStr">
+      <c r="I46" s="32" t="n">
+        <v>8700</v>
+      </c>
+      <c r="J46" s="32">
+        <f>I46*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="27.75" customHeight="1" s="23">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B46" s="25" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C46" s="25" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="inlineStr">
-        <is>
-          <t>Shinjuku Gyoen / Akihabara</t>
-        </is>
-      </c>
-      <c r="E46" s="25" t="n"/>
-      <c r="F46" s="25" t="n"/>
-      <c r="G46" s="25" t="n"/>
-      <c r="H46" s="25" t="n"/>
-      <c r="I46" s="26" t="n"/>
-      <c r="J46" s="26" t="n"/>
-    </row>
-    <row r="47" ht="27.75" customHeight="1" s="23">
-      <c r="A47" s="27" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B47" s="27" t="inlineStr">
-        <is>
-          <t>9 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C47" s="27" t="inlineStr">
-        <is>
-          <t>11:47</t>
-        </is>
-      </c>
-      <c r="D47" s="27" t="inlineStr">
-        <is>
-          <t>Zohor</t>
-        </is>
-      </c>
-      <c r="E47" s="27" t="inlineStr">
-        <is>
-          <t>Zohor 11:47</t>
-        </is>
-      </c>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-      <c r="I47" s="28" t="n"/>
-      <c r="J47" s="28" t="n"/>
+      <c r="C47" s="25" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="inlineStr">
+        <is>
+          <t>Drive Shinjuku → Kawaguchiko (Chuo Expressway → Kawaguchiko IC)</t>
+        </is>
+      </c>
+      <c r="E47" s="25" t="n"/>
+      <c r="F47" s="25" t="n"/>
+      <c r="G47" s="25" t="inlineStr">
+        <is>
+          <t>Tol ETC ~¥2,600 ÷ 6. ~1j30m kalau lancar — cuti panjang 3 hari, jangka 2j+</t>
+        </is>
+      </c>
+      <c r="H47" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I47" s="26" t="n">
+        <v>450</v>
+      </c>
+      <c r="J47" s="26">
+        <f>I47*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="27.75" customHeight="1" s="23">
       <c r="A48" s="25" t="inlineStr">
@@ -2220,65 +2237,69 @@
       </c>
       <c r="C48" s="25" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D48" s="25" t="inlineStr">
         <is>
-          <t>Lunch — halal</t>
+          <t>Chureito Pagoda — 398 anak tangga, Fuji paling jelas waktu pagi</t>
         </is>
       </c>
       <c r="E48" s="25" t="n"/>
-      <c r="F48" s="25" t="inlineStr">
+      <c r="F48" s="25" t="n"/>
+      <c r="G48" s="25" t="inlineStr">
+        <is>
+          <t>Parking Arakurayama Sengen Park (cepat penuh hujung minggu). Tangga mungkin berais</t>
+        </is>
+      </c>
+      <c r="H48" s="25" t="n"/>
+      <c r="I48" s="26" t="n"/>
+      <c r="J48" s="26" t="n"/>
+    </row>
+    <row r="49" ht="27.75" customHeight="1" s="23">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C49" s="25" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="inlineStr">
+        <is>
+          <t>Lunch — T&amp;T Fujiyama Halal Restaurant (hoto halal, mi tradisional Yamanashi)</t>
+        </is>
+      </c>
+      <c r="E49" s="25" t="n"/>
+      <c r="F49" s="25" t="inlineStr">
         <is>
           <t>Makan luar (halal)</t>
         </is>
       </c>
-      <c r="G48" s="25" t="n"/>
-      <c r="H48" s="25" t="inlineStr">
+      <c r="G49" s="25" t="inlineStr">
+        <is>
+          <t>Fujiyoshida, ~10min drive dari Chureito. Semua hoto ¥1,000. Buka 11:30-19:30</t>
+        </is>
+      </c>
+      <c r="H49" s="25" t="inlineStr">
         <is>
           <t>Food-Luar</t>
         </is>
       </c>
-      <c r="I48" s="26" t="n">
-        <v>1800</v>
-      </c>
-      <c r="J48" s="26">
-        <f>I48*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="27.75" customHeight="1" s="23">
-      <c r="A49" s="27" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B49" s="27" t="inlineStr">
-        <is>
-          <t>9 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C49" s="27" t="inlineStr">
-        <is>
-          <t>14:20</t>
-        </is>
-      </c>
-      <c r="D49" s="27" t="inlineStr">
-        <is>
-          <t>Asar</t>
-        </is>
-      </c>
-      <c r="E49" s="27" t="inlineStr">
-        <is>
-          <t>Asar 14:20</t>
-        </is>
-      </c>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="28" t="n"/>
-      <c r="J49" s="28" t="n"/>
+      <c r="I49" s="26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J49" s="26">
+        <f>I49*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="27.75" customHeight="1" s="23">
       <c r="A50" s="25" t="inlineStr">
@@ -2293,65 +2314,56 @@
       </c>
       <c r="C50" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>Shibuya Sky — slot 14:30 (OPTIONAL, boleh skip)</t>
-        </is>
-      </c>
-      <c r="E50" s="25" t="n"/>
+          <t>Zohor — Masjid Fujikawaguchiko (Funatsu, dekat stesen Kawaguchiko)</t>
+        </is>
+      </c>
+      <c r="E50" s="25" t="inlineStr">
+        <is>
+          <t>Zohor (masuk ~11:50)</t>
+        </is>
+      </c>
       <c r="F50" s="25" t="n"/>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>¥2,700 online (slot sebelum 15:00). Tiket buka 26 Dis 00:00. Keluar sebelum Maghrib ~16:45</t>
-        </is>
-      </c>
-      <c r="H50" s="25" t="inlineStr">
-        <is>
-          <t>Attraction-Optional</t>
-        </is>
-      </c>
-      <c r="I50" s="26" t="n">
-        <v>2700</v>
-      </c>
-      <c r="J50" s="26">
-        <f>I50*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+          <t>Masjid dibuka 2020, ada kafe halal dalam bangunan sama</t>
+        </is>
+      </c>
+      <c r="H50" s="25" t="n"/>
+      <c r="I50" s="26" t="n"/>
+      <c r="J50" s="26" t="n"/>
     </row>
     <row r="51" ht="27.75" customHeight="1" s="23">
-      <c r="A51" s="27" t="inlineStr">
+      <c r="A51" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B51" s="27" t="inlineStr">
+      <c r="B51" s="25" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C51" s="27" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="D51" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib</t>
-        </is>
-      </c>
-      <c r="E51" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib 16:45</t>
-        </is>
-      </c>
-      <c r="F51" s="27" t="n"/>
-      <c r="G51" s="27" t="n"/>
-      <c r="H51" s="27" t="n"/>
-      <c r="I51" s="28" t="n"/>
-      <c r="J51" s="28" t="n"/>
+      <c r="C51" s="25" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="inlineStr">
+        <is>
+          <t>Oishi Park — view Fuji dari seberang tasik Kawaguchiko (percuma)</t>
+        </is>
+      </c>
+      <c r="E51" s="25" t="n"/>
+      <c r="F51" s="25" t="n"/>
+      <c r="G51" s="25" t="n"/>
+      <c r="H51" s="25" t="n"/>
+      <c r="I51" s="26" t="n"/>
+      <c r="J51" s="26" t="n"/>
     </row>
     <row r="52" ht="27.75" customHeight="1" s="23">
       <c r="A52" s="25" t="inlineStr">
@@ -2366,65 +2378,56 @@
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="D52" s="25" t="inlineStr">
         <is>
-          <t>Dinner — halal (beli EXTRA utk bekal esok!)</t>
-        </is>
-      </c>
-      <c r="E52" s="25" t="n"/>
-      <c r="F52" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
+          <t>Asar</t>
+        </is>
+      </c>
+      <c r="E52" s="25" t="inlineStr">
+        <is>
+          <t>Asar ~14:15</t>
+        </is>
+      </c>
+      <c r="F52" s="25" t="n"/>
       <c r="G52" s="25" t="n"/>
-      <c r="H52" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I52" s="26" t="n">
-        <v>2200</v>
-      </c>
-      <c r="J52" s="26">
-        <f>I52*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="H52" s="25" t="n"/>
+      <c r="I52" s="26" t="n"/>
+      <c r="J52" s="26" t="n"/>
     </row>
     <row r="53" ht="27.75" customHeight="1" s="23">
-      <c r="A53" s="27" t="inlineStr">
+      <c r="A53" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B53" s="27" t="inlineStr">
+      <c r="B53" s="25" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C53" s="27" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="D53" s="27" t="inlineStr">
-        <is>
-          <t>Isyak</t>
-        </is>
-      </c>
-      <c r="E53" s="27" t="inlineStr">
-        <is>
-          <t>Isyak 18:05</t>
-        </is>
-      </c>
-      <c r="F53" s="27" t="n"/>
-      <c r="G53" s="27" t="n"/>
-      <c r="H53" s="27" t="n"/>
-      <c r="I53" s="28" t="n"/>
-      <c r="J53" s="28" t="n"/>
+      <c r="C53" s="25" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="inlineStr">
+        <is>
+          <t>Oshino Hakkai — 8 kolam air mata air Fuji (percuma), ~25min drive</t>
+        </is>
+      </c>
+      <c r="E53" s="25" t="n"/>
+      <c r="F53" s="25" t="n"/>
+      <c r="G53" s="25" t="inlineStr">
+        <is>
+          <t>Air salji Fuji ditapis lava berpuluh tahun — boleh isi botol &amp; minum</t>
+        </is>
+      </c>
+      <c r="H53" s="25" t="n"/>
+      <c r="I53" s="26" t="n"/>
+      <c r="J53" s="26" t="n"/>
     </row>
     <row r="54" ht="27.75" customHeight="1" s="23">
       <c r="A54" s="25" t="inlineStr">
@@ -2439,33 +2442,24 @@
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="D54" s="25" t="inlineStr">
         <is>
-          <t>Beli bekal halal utk esok (Kawaguchiko takde halal food)</t>
-        </is>
-      </c>
-      <c r="E54" s="25" t="n"/>
-      <c r="F54" s="25" t="inlineStr">
-        <is>
-          <t>Bekal</t>
-        </is>
-      </c>
+          <t>Maghrib — Masjid Fujikawaguchiko</t>
+        </is>
+      </c>
+      <c r="E54" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib ~16:45</t>
+        </is>
+      </c>
+      <c r="F54" s="25" t="n"/>
       <c r="G54" s="25" t="n"/>
-      <c r="H54" s="25" t="inlineStr">
-        <is>
-          <t>Food-Bekal</t>
-        </is>
-      </c>
-      <c r="I54" s="26" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J54" s="26">
-        <f>I54*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="H54" s="25" t="n"/>
+      <c r="I54" s="26" t="n"/>
+      <c r="J54" s="26" t="n"/>
     </row>
     <row r="55" ht="27.75" customHeight="1" s="23">
       <c r="A55" s="25" t="inlineStr">
@@ -2480,24 +2474,28 @@
       </c>
       <c r="C55" s="25" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="D55" s="25" t="inlineStr">
         <is>
-          <t>Check-in manga cafe</t>
+          <t>Dinner — Halal food and cafe (Masjid) / Idaten Bettei (halal, dekat stesen)</t>
         </is>
       </c>
       <c r="E55" s="25" t="n"/>
-      <c r="F55" s="25" t="n"/>
+      <c r="F55" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
       <c r="G55" s="25" t="n"/>
       <c r="H55" s="25" t="inlineStr">
         <is>
-          <t>Accommodation</t>
+          <t>Food-Luar</t>
         </is>
       </c>
       <c r="I55" s="26" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="J55" s="26">
         <f>I55*'Budget Summary'!$B$2</f>
@@ -2505,307 +2503,342 @@
       </c>
     </row>
     <row r="56" ht="27.75" customHeight="1" s="23">
-      <c r="A56" s="27" t="inlineStr">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C56" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="inlineStr">
+        <is>
+          <t>Isyak — Masjid Fujikawaguchiko</t>
+        </is>
+      </c>
+      <c r="E56" s="25" t="inlineStr">
+        <is>
+          <t>Isyak ~18:00</t>
+        </is>
+      </c>
+      <c r="F56" s="25" t="n"/>
+      <c r="G56" s="25" t="n"/>
+      <c r="H56" s="25" t="n"/>
+      <c r="I56" s="26" t="n"/>
+      <c r="J56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="27.75" customHeight="1" s="23">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C57" s="25" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="inlineStr">
+        <is>
+          <t>Isi minyak + konbini: snek malam, sarapan esok, kairo, air</t>
+        </is>
+      </c>
+      <c r="E57" s="25" t="n"/>
+      <c r="F57" s="25" t="inlineStr">
+        <is>
+          <t>Snek/Bekal</t>
+        </is>
+      </c>
+      <c r="G57" s="25" t="n"/>
+      <c r="H57" s="25" t="inlineStr">
+        <is>
+          <t>Food-Bekal</t>
+        </is>
+      </c>
+      <c r="I57" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="J57" s="26">
+        <f>I57*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="27.75" customHeight="1" s="23">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C58" s="31" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D58" s="31" t="inlineStr">
+        <is>
+          <t>TIDUR DALAM KERETA — Michi-no-eki Katsuyama (tepi tasik, parking percuma, tandas 24j)</t>
+        </is>
+      </c>
+      <c r="E58" s="31" t="n"/>
+      <c r="F58" s="31" t="n"/>
+      <c r="G58" s="31" t="inlineStr">
+        <is>
+          <t>SUHU purata −7°C (boleh −10°C). Enjin MATI masa semua tidur; salji boleh tutup ekzos → karbon monoksida. Sleeping bag −10°C + kairo + CO detector. JANGAN guna dapur gas</t>
+        </is>
+      </c>
+      <c r="H58" s="31" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="I58" s="32" t="n"/>
+      <c r="J58" s="32" t="n"/>
+    </row>
+    <row r="59" ht="27.75" customHeight="1" s="23">
+      <c r="A59" s="27" t="inlineStr">
         <is>
           <t>5
 (Ahad)</t>
         </is>
       </c>
-      <c r="B56" s="27" t="inlineStr">
+      <c r="B59" s="27" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C56" s="27" t="inlineStr">
+      <c r="C59" s="27" t="inlineStr">
         <is>
           <t>05:22</t>
         </is>
       </c>
-      <c r="D56" s="27" t="inlineStr">
-        <is>
-          <t>Subuh</t>
-        </is>
-      </c>
-      <c r="E56" s="27" t="inlineStr">
-        <is>
-          <t>Subuh 05:22</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n"/>
-      <c r="G56" s="27" t="n"/>
-      <c r="H56" s="27" t="n"/>
-      <c r="I56" s="28" t="n"/>
-      <c r="J56" s="28" t="n"/>
-    </row>
-    <row r="57" ht="27.75" customHeight="1" s="23">
-      <c r="A57" s="25" t="inlineStr">
+      <c r="D59" s="27" t="inlineStr">
+        <is>
+          <t>Subuh (Michi-no-eki / tepi tasik — bawa sejadah)</t>
+        </is>
+      </c>
+      <c r="E59" s="27" t="inlineStr">
+        <is>
+          <t>Subuh ~05:22</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n"/>
+      <c r="G59" s="27" t="n"/>
+      <c r="H59" s="27" t="n"/>
+      <c r="I59" s="28" t="n"/>
+      <c r="J59" s="28" t="n"/>
+    </row>
+    <row r="60" ht="27.75" customHeight="1" s="23">
+      <c r="A60" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B57" s="25" t="inlineStr">
+      <c r="B60" s="25" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C57" s="25" t="inlineStr">
+      <c r="C60" s="25" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D57" s="25" t="inlineStr">
-        <is>
-          <t>Breakfast — bekal/conbini</t>
-        </is>
-      </c>
-      <c r="E57" s="25" t="n"/>
-      <c r="F57" s="25" t="inlineStr">
+      <c r="D60" s="25" t="inlineStr">
+        <is>
+          <t>Matahari terbit + Fuji — Oishi Park / tepi tasik (~06:50)</t>
+        </is>
+      </c>
+      <c r="E60" s="25" t="n"/>
+      <c r="F60" s="25" t="n"/>
+      <c r="G60" s="25" t="inlineStr">
+        <is>
+          <t>Pagi = Fuji paling jelas, tasik paling tenang</t>
+        </is>
+      </c>
+      <c r="H60" s="25" t="n"/>
+      <c r="I60" s="26" t="n"/>
+      <c r="J60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="27.75" customHeight="1" s="23">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B61" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C61" s="25" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D61" s="25" t="inlineStr">
+        <is>
+          <t>Breakfast — snek/konbini</t>
+        </is>
+      </c>
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="25" t="inlineStr">
         <is>
           <t>Makan luar (halal)</t>
         </is>
       </c>
-      <c r="G57" s="25" t="n"/>
-      <c r="H57" s="25" t="inlineStr">
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="25" t="inlineStr">
         <is>
           <t>Food-Luar</t>
         </is>
       </c>
-      <c r="I57" s="26" t="n">
+      <c r="I61" s="26" t="n">
         <v>600</v>
       </c>
-      <c r="J57" s="26">
-        <f>I57*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="27.75" customHeight="1" s="23">
-      <c r="A58" s="25" t="inlineStr">
+      <c r="J61" s="26">
+        <f>I61*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="27.75" customHeight="1" s="23">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B58" s="25" t="inlineStr">
+      <c r="B62" s="25" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C58" s="25" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="inlineStr">
-        <is>
-          <t>Bas Shinjuku → Kawaguchiko</t>
-        </is>
-      </c>
-      <c r="E58" s="25" t="n"/>
-      <c r="F58" s="25" t="n"/>
-      <c r="G58" s="25" t="inlineStr">
-        <is>
-          <t>Highway bus, ¥2,000-2,200, ~1j45m</t>
-        </is>
-      </c>
-      <c r="H58" s="25" t="inlineStr">
+      <c r="C62" s="25" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D62" s="25" t="inlineStr">
+        <is>
+          <t>Drive balik Kawaguchiko → Shinjuku</t>
+        </is>
+      </c>
+      <c r="E62" s="25" t="n"/>
+      <c r="F62" s="25" t="n"/>
+      <c r="G62" s="25" t="inlineStr">
+        <is>
+          <t>Tol ETC ~¥2,600 ÷ 6. Ahad pagi arah Tokyo biasanya lancar (orang balik Isnin)</t>
+        </is>
+      </c>
+      <c r="H62" s="25" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="I58" s="26" t="n">
-        <v>2100</v>
-      </c>
-      <c r="J58" s="26">
-        <f>I58*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="27.75" customHeight="1" s="23">
-      <c r="A59" s="25" t="inlineStr">
+      <c r="I62" s="26" t="n">
+        <v>450</v>
+      </c>
+      <c r="J62" s="26">
+        <f>I62*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="27.75" customHeight="1" s="23">
+      <c r="A63" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B59" s="25" t="inlineStr">
+      <c r="B63" s="31" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>09:45</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="inlineStr">
-        <is>
-          <t>Sampai Kawaguchiko — spot Fuji (Chureito Pagoda/Lake)</t>
-        </is>
-      </c>
-      <c r="E59" s="25" t="n"/>
-      <c r="F59" s="25" t="n"/>
-      <c r="G59" s="25" t="n"/>
-      <c r="H59" s="25" t="n"/>
-      <c r="I59" s="26" t="n"/>
-      <c r="J59" s="26" t="n"/>
-    </row>
-    <row r="60" ht="27.75" customHeight="1" s="23">
-      <c r="A60" s="27" t="inlineStr">
+      <c r="C63" s="31" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D63" s="31" t="inlineStr">
+        <is>
+          <t>Isi minyak penuh &amp; PULANGKAN KERETA (Shinjuku)</t>
+        </is>
+      </c>
+      <c r="E63" s="31" t="n"/>
+      <c r="F63" s="31" t="n"/>
+      <c r="G63" s="31" t="inlineStr">
+        <is>
+          <t>Minyak ~¥5k + parking ~¥1k ÷ 6. Lewat pulang = caj ~¥2,860/jam. Bagasi masuk coin locker Busta Shinjuku</t>
+        </is>
+      </c>
+      <c r="H63" s="31" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I63" s="32" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J63" s="32">
+        <f>I63*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="27.75" customHeight="1" s="23">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B60" s="27" t="inlineStr">
+      <c r="B64" s="25" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C60" s="27" t="inlineStr">
-        <is>
-          <t>11:50</t>
-        </is>
-      </c>
-      <c r="D60" s="27" t="inlineStr">
-        <is>
-          <t>Zohor (luar — bawa sejadah + kompas kiblat app)</t>
-        </is>
-      </c>
-      <c r="E60" s="27" t="inlineStr">
-        <is>
-          <t>Zohor ~11:50</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n"/>
-      <c r="G60" s="27" t="n"/>
-      <c r="H60" s="27" t="n"/>
-      <c r="I60" s="28" t="n"/>
-      <c r="J60" s="28" t="n"/>
-    </row>
-    <row r="61" ht="27.75" customHeight="1" s="23">
-      <c r="A61" s="31" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B61" s="31" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C61" s="31" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="D61" s="31" t="inlineStr">
-        <is>
-          <t>Lunch — bekal yang dibawa dari Tokyo</t>
-        </is>
-      </c>
-      <c r="E61" s="31" t="n"/>
-      <c r="F61" s="31" t="inlineStr">
-        <is>
-          <t>Bekal (dah dibeli)</t>
-        </is>
-      </c>
-      <c r="G61" s="31" t="inlineStr">
-        <is>
-          <t>TAKDE halal food kat Kawaguchiko</t>
-        </is>
-      </c>
-      <c r="H61" s="31" t="n"/>
-      <c r="I61" s="32" t="n"/>
-      <c r="J61" s="32" t="n"/>
-    </row>
-    <row r="62" ht="27.75" customHeight="1" s="23">
-      <c r="A62" s="27" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B62" s="27" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C62" s="27" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="D62" s="27" t="inlineStr">
-        <is>
-          <t>Asar</t>
-        </is>
-      </c>
-      <c r="E62" s="27" t="inlineStr">
-        <is>
-          <t>Asar ~14:15</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n"/>
-      <c r="G62" s="27" t="n"/>
-      <c r="H62" s="27" t="n"/>
-      <c r="I62" s="28" t="n"/>
-      <c r="J62" s="28" t="n"/>
-    </row>
-    <row r="63" ht="27.75" customHeight="1" s="23">
-      <c r="A63" s="25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B63" s="25" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C63" s="25" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D63" s="25" t="inlineStr">
-        <is>
-          <t>Explore lagi / gambar area lake</t>
-        </is>
-      </c>
-      <c r="E63" s="25" t="n"/>
-      <c r="F63" s="25" t="n"/>
-      <c r="G63" s="25" t="n"/>
-      <c r="H63" s="25" t="n"/>
-      <c r="I63" s="26" t="n"/>
-      <c r="J63" s="26" t="n"/>
-    </row>
-    <row r="64" ht="27.75" customHeight="1" s="23">
-      <c r="A64" s="27" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B64" s="27" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C64" s="27" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="D64" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib (view Fuji + sunset)</t>
-        </is>
-      </c>
-      <c r="E64" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib ~16:45</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n"/>
-      <c r="G64" s="27" t="n"/>
-      <c r="H64" s="27" t="n"/>
-      <c r="I64" s="28" t="n"/>
-      <c r="J64" s="28" t="n"/>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="inlineStr">
+        <is>
+          <t>Local transport Tokyo (metro/IC card)</t>
+        </is>
+      </c>
+      <c r="E64" s="25" t="n"/>
+      <c r="F64" s="25" t="n"/>
+      <c r="G64" s="25" t="inlineStr">
+        <is>
+          <t>~¥800/hari</t>
+        </is>
+      </c>
+      <c r="H64" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I64" s="26" t="n">
+        <v>800</v>
+      </c>
+      <c r="J64" s="26">
+        <f>I64*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="27.75" customHeight="1" s="23">
       <c r="A65" s="25" t="inlineStr">
@@ -2820,65 +2853,65 @@
       </c>
       <c r="C65" s="25" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>11:47</t>
         </is>
       </c>
       <c r="D65" s="25" t="inlineStr">
         <is>
-          <t>Dinner — snack/bekal tambahan (beli kat konbini stesen)</t>
-        </is>
-      </c>
-      <c r="E65" s="25" t="n"/>
-      <c r="F65" s="25" t="inlineStr">
-        <is>
-          <t>Snack/Bekal</t>
-        </is>
-      </c>
+          <t>Zohor</t>
+        </is>
+      </c>
+      <c r="E65" s="25" t="inlineStr">
+        <is>
+          <t>Zohor 11:47</t>
+        </is>
+      </c>
+      <c r="F65" s="25" t="n"/>
       <c r="G65" s="25" t="n"/>
-      <c r="H65" s="25" t="inlineStr">
+      <c r="H65" s="25" t="n"/>
+      <c r="I65" s="26" t="n"/>
+      <c r="J65" s="26" t="n"/>
+    </row>
+    <row r="66" ht="27.75" customHeight="1" s="23">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>Lunch — halal (Shinjuku/Shibuya)</t>
+        </is>
+      </c>
+      <c r="E66" s="25" t="n"/>
+      <c r="F66" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G66" s="25" t="n"/>
+      <c r="H66" s="25" t="inlineStr">
         <is>
           <t>Food-Luar</t>
         </is>
       </c>
-      <c r="I65" s="26" t="n">
-        <v>800</v>
-      </c>
-      <c r="J65" s="26">
-        <f>I65*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="27.75" customHeight="1" s="23">
-      <c r="A66" s="27" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B66" s="27" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C66" s="27" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D66" s="27" t="inlineStr">
-        <is>
-          <t>Isyak</t>
-        </is>
-      </c>
-      <c r="E66" s="27" t="inlineStr">
-        <is>
-          <t>Isyak ~18:00</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n"/>
-      <c r="G66" s="27" t="n"/>
-      <c r="H66" s="27" t="n"/>
-      <c r="I66" s="28" t="n"/>
-      <c r="J66" s="28" t="n"/>
+      <c r="I66" s="26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="J66" s="26">
+        <f>I66*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="27.75" customHeight="1" s="23">
       <c r="A67" s="25" t="inlineStr">
@@ -2893,89 +2926,92 @@
       </c>
       <c r="C67" s="25" t="inlineStr">
         <is>
-          <t>20:47</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="D67" s="25" t="inlineStr">
         <is>
-          <t>Bas overnight Kawaguchiko → Osaka (tidur atas bas)</t>
-        </is>
-      </c>
-      <c r="E67" s="25" t="n"/>
+          <t>Asar</t>
+        </is>
+      </c>
+      <c r="E67" s="25" t="inlineStr">
+        <is>
+          <t>Asar 14:20</t>
+        </is>
+      </c>
       <c r="F67" s="25" t="n"/>
-      <c r="G67" s="25" t="inlineStr">
-        <is>
-          <t>Fujiyama Liner (Fujikyu), ¥6,700-8,700, ~10j</t>
-        </is>
-      </c>
-      <c r="H67" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I67" s="26" t="n">
-        <v>7700</v>
-      </c>
-      <c r="J67" s="26">
-        <f>I67*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="G67" s="25" t="n"/>
+      <c r="H67" s="25" t="n"/>
+      <c r="I67" s="26" t="n"/>
+      <c r="J67" s="26" t="n"/>
     </row>
     <row r="68" ht="27.75" customHeight="1" s="23">
-      <c r="A68" s="27" t="inlineStr">
-        <is>
-          <t>6
-(Isnin)</t>
-        </is>
-      </c>
-      <c r="B68" s="27" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C68" s="27" t="inlineStr">
-        <is>
-          <t>~05:38</t>
-        </is>
-      </c>
-      <c r="D68" s="27" t="inlineStr">
-        <is>
-          <t>Subuh (atas bas — anggar kiblat)</t>
-        </is>
-      </c>
-      <c r="E68" s="27" t="inlineStr">
-        <is>
-          <t>Subuh ~05:38</t>
-        </is>
-      </c>
-      <c r="F68" s="27" t="n"/>
-      <c r="G68" s="27" t="n"/>
-      <c r="H68" s="27" t="n"/>
-      <c r="I68" s="28" t="n"/>
-      <c r="J68" s="28" t="n"/>
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B68" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C68" s="25" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D68" s="25" t="inlineStr">
+        <is>
+          <t>Shibuya Sky — slot 14:30 (OPTIONAL, boleh skip)</t>
+        </is>
+      </c>
+      <c r="E68" s="25" t="n"/>
+      <c r="F68" s="25" t="n"/>
+      <c r="G68" s="25" t="inlineStr">
+        <is>
+          <t>¥2,700 online. Tiket untuk Ahad 10 Jan buka 27 Dis 00:00. Keluar sebelum Maghrib ~16:45</t>
+        </is>
+      </c>
+      <c r="H68" s="25" t="inlineStr">
+        <is>
+          <t>Attraction-Optional</t>
+        </is>
+      </c>
+      <c r="I68" s="26" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J68" s="26">
+        <f>I68*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="27.75" customHeight="1" s="23">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>11 Jan 2027</t>
+          <t>10 Jan 2027</t>
         </is>
       </c>
       <c r="C69" s="25" t="inlineStr">
         <is>
-          <t>06:53</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="D69" s="25" t="inlineStr">
         <is>
-          <t>Sampai Osaka → terus balik guesthouse, mandi, tidur sekejap</t>
-        </is>
-      </c>
-      <c r="E69" s="25" t="n"/>
+          <t>Maghrib — surau Shibuya PARCO 5F</t>
+        </is>
+      </c>
+      <c r="E69" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib 16:45</t>
+        </is>
+      </c>
       <c r="F69" s="25" t="n"/>
       <c r="G69" s="25" t="n"/>
       <c r="H69" s="25" t="n"/>
@@ -2985,38 +3021,42 @@
     <row r="70" ht="27.75" customHeight="1" s="23">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>11 Jan 2027</t>
+          <t>10 Jan 2027</t>
         </is>
       </c>
       <c r="C70" s="25" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>Breakfast — masak kat guesthouse</t>
+          <t>Akihabara + dinner halal (Halal Wagyu Karemen King)</t>
         </is>
       </c>
       <c r="E70" s="25" t="n"/>
       <c r="F70" s="25" t="inlineStr">
         <is>
-          <t>Masak</t>
-        </is>
-      </c>
-      <c r="G70" s="25" t="n"/>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G70" s="25" t="inlineStr">
+        <is>
+          <t>Masjid Nusantara ~4min dari Karemen King</t>
+        </is>
+      </c>
       <c r="H70" s="25" t="inlineStr">
         <is>
-          <t>Food-Masak</t>
+          <t>Food-Luar</t>
         </is>
       </c>
       <c r="I70" s="26" t="n">
-        <v>600</v>
+        <v>2200</v>
       </c>
       <c r="J70" s="26">
         <f>I70*'Budget Summary'!$B$2</f>
@@ -3024,72 +3064,59 @@
       </c>
     </row>
     <row r="71" ht="27.75" customHeight="1" s="23">
-      <c r="A71" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B71" s="29" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C71" s="29" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D71" s="29" t="inlineStr">
-        <is>
-          <t>Gerak ke Kyoto: Midosuji Namba → Yodoyabashi, tukar Keihan → Kiyomizu-Gojo</t>
-        </is>
-      </c>
-      <c r="E71" s="29" t="n"/>
-      <c r="F71" s="29" t="n"/>
-      <c r="G71" s="29" t="inlineStr">
-        <is>
-          <t>¥240 + ¥430, ~1j15m. Isnin 11 Jan = CUTI UMUM Jepun (Seijin no Hi), Kyoto sesak</t>
-        </is>
-      </c>
-      <c r="H71" s="29" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I71" s="30" t="n">
-        <v>670</v>
-      </c>
-      <c r="J71" s="30">
-        <f>I71*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="A71" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B71" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C71" s="25" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="D71" s="25" t="inlineStr">
+        <is>
+          <t>Isyak (Masjid Nusantara, Akihabara)</t>
+        </is>
+      </c>
+      <c r="E71" s="25" t="inlineStr">
+        <is>
+          <t>Isyak 18:05</t>
+        </is>
+      </c>
+      <c r="F71" s="25" t="n"/>
+      <c r="G71" s="25" t="n"/>
+      <c r="H71" s="25" t="n"/>
+      <c r="I71" s="26" t="n"/>
+      <c r="J71" s="26" t="n"/>
     </row>
     <row r="72" ht="27.75" customHeight="1" s="23">
       <c r="A72" s="25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B72" s="25" t="inlineStr">
         <is>
-          <t>11 Jan 2027</t>
+          <t>10 Jan 2027</t>
         </is>
       </c>
       <c r="C72" s="25" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D72" s="25" t="inlineStr">
         <is>
-          <t>Zohor — surau Curry Club Ruu, Ninenzaka (ada tempat wuduk, muat 4-5 orang, solat 2 giliran)</t>
-        </is>
-      </c>
-      <c r="E72" s="25" t="inlineStr">
-        <is>
-          <t>Zohor 12:00</t>
-        </is>
-      </c>
+          <t>Ambil bagasi dari coin locker, ke Busta Shinjuku</t>
+        </is>
+      </c>
+      <c r="E72" s="25" t="n"/>
       <c r="F72" s="25" t="n"/>
       <c r="G72" s="25" t="n"/>
       <c r="H72" s="25" t="n"/>
@@ -3097,268 +3124,265 @@
       <c r="J72" s="26" t="n"/>
     </row>
     <row r="73" ht="27.75" customHeight="1" s="23">
-      <c r="A73" s="27" t="inlineStr">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B73" s="31" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C73" s="31" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D73" s="31" t="inlineStr">
+        <is>
+          <t>Bas overnight Tokyo (Busta Shinjuku) → Osaka (tidur atas bas)</t>
+        </is>
+      </c>
+      <c r="E73" s="31" t="n"/>
+      <c r="F73" s="31" t="n"/>
+      <c r="G73" s="31" t="inlineStr">
+        <is>
+          <t>Willer Express ~¥3,000-5,000, ~8-10j. Ahad cuti panjang — book awal</t>
+        </is>
+      </c>
+      <c r="H73" s="31" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J73" s="32">
+        <f>I73*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="27.75" customHeight="1" s="23">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>6
+(Isnin)</t>
+        </is>
+      </c>
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C74" s="27" t="inlineStr">
+        <is>
+          <t>~05:38</t>
+        </is>
+      </c>
+      <c r="D74" s="27" t="inlineStr">
+        <is>
+          <t>Subuh (atas bas — anggar kiblat)</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr">
+        <is>
+          <t>Subuh ~05:38</t>
+        </is>
+      </c>
+      <c r="F74" s="27" t="n"/>
+      <c r="G74" s="27" t="n"/>
+      <c r="H74" s="27" t="n"/>
+      <c r="I74" s="28" t="n"/>
+      <c r="J74" s="28" t="n"/>
+    </row>
+    <row r="75" ht="27.75" customHeight="1" s="23">
+      <c r="A75" s="25" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B73" s="27" t="inlineStr">
+      <c r="B75" s="25" t="inlineStr">
         <is>
           <t>11 Jan 2027</t>
         </is>
       </c>
-      <c r="C73" s="27" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="D73" s="27" t="inlineStr">
-        <is>
-          <t>Lunch — Curry Club Ruu Ninenzaka (kari Jepun halal)</t>
-        </is>
-      </c>
-      <c r="E73" s="27" t="n"/>
-      <c r="F73" s="27" t="inlineStr">
+      <c r="C75" s="25" t="inlineStr">
+        <is>
+          <t>~07:30</t>
+        </is>
+      </c>
+      <c r="D75" s="25" t="inlineStr">
+        <is>
+          <t>Sampai Osaka (bas malam Willer, ~07:00-09:00) → terus balik guesthouse, mandi, tidur sekejap</t>
+        </is>
+      </c>
+      <c r="E75" s="25" t="n"/>
+      <c r="F75" s="25" t="n"/>
+      <c r="G75" s="25" t="n"/>
+      <c r="H75" s="25" t="n"/>
+      <c r="I75" s="26" t="n"/>
+      <c r="J75" s="26" t="n"/>
+    </row>
+    <row r="76" ht="27.75" customHeight="1" s="23">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D76" s="29" t="inlineStr">
+        <is>
+          <t>Breakfast — masak kat guesthouse</t>
+        </is>
+      </c>
+      <c r="E76" s="29" t="n"/>
+      <c r="F76" s="29" t="inlineStr">
+        <is>
+          <t>Masak</t>
+        </is>
+      </c>
+      <c r="G76" s="29" t="n"/>
+      <c r="H76" s="29" t="inlineStr">
+        <is>
+          <t>Food-Masak</t>
+        </is>
+      </c>
+      <c r="I76" s="30" t="n">
+        <v>600</v>
+      </c>
+      <c r="J76" s="30">
+        <f>I76*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="27.75" customHeight="1" s="23">
+      <c r="A77" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B77" s="25" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C77" s="25" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D77" s="25" t="inlineStr">
+        <is>
+          <t>Gerak ke Kyoto: Midosuji Namba → Yodoyabashi, tukar Keihan → Kiyomizu-Gojo</t>
+        </is>
+      </c>
+      <c r="E77" s="25" t="n"/>
+      <c r="F77" s="25" t="n"/>
+      <c r="G77" s="25" t="inlineStr">
+        <is>
+          <t>¥240 + ¥430, ~1j15m. Isnin 11 Jan = CUTI UMUM Jepun (Seijin no Hi), Kyoto sesak</t>
+        </is>
+      </c>
+      <c r="H77" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I77" s="26" t="n">
+        <v>670</v>
+      </c>
+      <c r="J77" s="26">
+        <f>I77*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" ht="27.75" customHeight="1" s="23">
+      <c r="A78" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B78" s="25" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C78" s="25" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="inlineStr">
+        <is>
+          <t>Zohor — ruang solat Shinjuku-tei Kiyomizu (restoran buka 12:00)</t>
+        </is>
+      </c>
+      <c r="E78" s="25" t="inlineStr">
+        <is>
+          <t>Zohor 12:00</t>
+        </is>
+      </c>
+      <c r="F78" s="25" t="n"/>
+      <c r="G78" s="25" t="n"/>
+      <c r="H78" s="25" t="n"/>
+      <c r="I78" s="26" t="n"/>
+      <c r="J78" s="26" t="n"/>
+    </row>
+    <row r="79" ht="27.75" customHeight="1" s="23">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B79" s="25" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C79" s="25" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D79" s="25" t="inlineStr">
+        <is>
+          <t>Lunch — HALAL WAGYU RAMEN SHINJUKU-TEI Kiyomizu (halal, ada ruang solat)</t>
+        </is>
+      </c>
+      <c r="E79" s="25" t="n"/>
+      <c r="F79" s="25" t="inlineStr">
         <is>
           <t>Makan luar (halal)</t>
         </is>
       </c>
-      <c r="G73" s="27" t="inlineStr">
-        <is>
-          <t>~10min jalan kaki ke Kiyomizu-dera</t>
-        </is>
-      </c>
-      <c r="H73" s="27" t="inlineStr">
+      <c r="G79" s="25" t="inlineStr">
+        <is>
+          <t>148 Hoshinocho, dekat Ninenzaka. Chicken paitan ¥1,500-2,500; wagyu ramen ¥4,500. Backup: Halal Ramen Honolu Premier, Gion (buka 11:30)</t>
+        </is>
+      </c>
+      <c r="H79" s="25" t="inlineStr">
         <is>
           <t>Food-Luar</t>
         </is>
       </c>
-      <c r="I73" s="28" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J73" s="28">
-        <f>I73*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" ht="27.75" customHeight="1" s="23">
-      <c r="A74" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B74" s="29" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C74" s="29" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="D74" s="29" t="inlineStr">
-        <is>
-          <t>Kiyomizu-dera (jalan naik Ninenzaka/Sannenzaka)</t>
-        </is>
-      </c>
-      <c r="E74" s="29" t="n"/>
-      <c r="F74" s="29" t="n"/>
-      <c r="G74" s="29" t="inlineStr">
-        <is>
-          <t>¥500, bayar TUNAI. Buka 06:00-18:00. Jalan dari stesen curam ~25min; teksi kongsi 6 orang pun murah</t>
-        </is>
-      </c>
-      <c r="H74" s="29" t="inlineStr">
-        <is>
-          <t>Attraction-Optional</t>
-        </is>
-      </c>
-      <c r="I74" s="30" t="n">
-        <v>500</v>
-      </c>
-      <c r="J74" s="30">
-        <f>I74*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" ht="27.75" customHeight="1" s="23">
-      <c r="A75" s="27" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B75" s="27" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C75" s="27" t="inlineStr">
-        <is>
-          <t>14:35</t>
-        </is>
-      </c>
-      <c r="D75" s="27" t="inlineStr">
-        <is>
-          <t>Asar (kawasan Kiyomizu / surau restoran halal berdekatan)</t>
-        </is>
-      </c>
-      <c r="E75" s="27" t="inlineStr">
-        <is>
-          <t>Asar 14:35</t>
-        </is>
-      </c>
-      <c r="F75" s="27" t="n"/>
-      <c r="G75" s="27" t="n"/>
-      <c r="H75" s="27" t="n"/>
-      <c r="I75" s="28" t="n"/>
-      <c r="J75" s="28" t="n"/>
-    </row>
-    <row r="76" ht="27.75" customHeight="1" s="23">
-      <c r="A76" s="25" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B76" s="25" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C76" s="25" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="D76" s="25" t="inlineStr">
-        <is>
-          <t>Balik Osaka: Keihan Kiyomizu-Gojo → Yodoyabashi → Midosuji → Namba</t>
-        </is>
-      </c>
-      <c r="E76" s="25" t="n"/>
-      <c r="F76" s="25" t="n"/>
-      <c r="G76" s="25" t="inlineStr">
-        <is>
-          <t>¥430 + ¥240, ~1j15m. Sampai Namba ~16:45</t>
-        </is>
-      </c>
-      <c r="H76" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I76" s="26" t="n">
-        <v>670</v>
-      </c>
-      <c r="J76" s="26">
-        <f>I76*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="27.75" customHeight="1" s="23">
-      <c r="A77" s="27" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B77" s="27" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C77" s="27" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="D77" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib</t>
-        </is>
-      </c>
-      <c r="E77" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib 17:00</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
-      <c r="H77" s="27" t="n"/>
-      <c r="I77" s="28" t="n"/>
-      <c r="J77" s="28" t="n"/>
-    </row>
-    <row r="78" ht="27.75" customHeight="1" s="23">
-      <c r="A78" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B78" s="29" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="D78" s="29" t="inlineStr">
-        <is>
-          <t>Dinner — masak (habiskan baki bahan)</t>
-        </is>
-      </c>
-      <c r="E78" s="29" t="n"/>
-      <c r="F78" s="29" t="inlineStr">
-        <is>
-          <t>Masak</t>
-        </is>
-      </c>
-      <c r="G78" s="29" t="n"/>
-      <c r="H78" s="29" t="inlineStr">
-        <is>
-          <t>Food-Masak</t>
-        </is>
-      </c>
-      <c r="I78" s="30" t="n">
-        <v>700</v>
-      </c>
-      <c r="J78" s="30">
-        <f>I78*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" ht="27.75" customHeight="1" s="23">
-      <c r="A79" s="27" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B79" s="27" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C79" s="27" t="inlineStr">
-        <is>
-          <t>18:20</t>
-        </is>
-      </c>
-      <c r="D79" s="27" t="inlineStr">
-        <is>
-          <t>Isyak</t>
-        </is>
-      </c>
-      <c r="E79" s="27" t="inlineStr">
-        <is>
-          <t>Isyak 18:20</t>
-        </is>
-      </c>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
-      <c r="H79" s="27" t="n"/>
-      <c r="I79" s="28" t="n"/>
-      <c r="J79" s="28" t="n"/>
+      <c r="I79" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J79" s="26">
+        <f>I79*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="80" ht="27.75" customHeight="1" s="23">
       <c r="A80" s="25" t="inlineStr">
@@ -3373,44 +3397,60 @@
       </c>
       <c r="C80" s="25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D80" s="25" t="inlineStr">
         <is>
-          <t>Kemas beg, tidur awal (flight awal esok!)</t>
+          <t>Kiyomizu-dera (jalan naik Ninenzaka/Sannenzaka)</t>
         </is>
       </c>
       <c r="E80" s="25" t="n"/>
       <c r="F80" s="25" t="n"/>
-      <c r="G80" s="25" t="n"/>
-      <c r="H80" s="25" t="n"/>
-      <c r="I80" s="26" t="n"/>
-      <c r="J80" s="26" t="n"/>
+      <c r="G80" s="25" t="inlineStr">
+        <is>
+          <t>¥500, bayar TUNAI. Buka 06:00-18:00. Jalan dari stesen curam ~25min; teksi kongsi 6 orang pun murah</t>
+        </is>
+      </c>
+      <c r="H80" s="25" t="inlineStr">
+        <is>
+          <t>Attraction-Optional</t>
+        </is>
+      </c>
+      <c r="I80" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="J80" s="26">
+        <f>I80*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="81" ht="27.75" customHeight="1" s="23">
       <c r="A81" s="25" t="inlineStr">
         <is>
-          <t>7
-(Selasa)</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C81" s="25" t="inlineStr">
         <is>
-          <t>~04:30</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="D81" s="25" t="inlineStr">
         <is>
-          <t>Bangun awal</t>
-        </is>
-      </c>
-      <c r="E81" s="25" t="n"/>
+          <t>Asar (kawasan Kiyomizu / surau restoran halal berdekatan)</t>
+        </is>
+      </c>
+      <c r="E81" s="25" t="inlineStr">
+        <is>
+          <t>Asar 14:35</t>
+        </is>
+      </c>
       <c r="F81" s="25" t="n"/>
       <c r="G81" s="25" t="n"/>
       <c r="H81" s="25" t="n"/>
@@ -3420,29 +3460,29 @@
     <row r="82" ht="27.75" customHeight="1" s="23">
       <c r="A82" s="25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C82" s="25" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D82" s="25" t="inlineStr">
         <is>
-          <t>Nankai Airport Express Namba → KIX</t>
+          <t>Balik Osaka: Keihan Kiyomizu-Gojo → Yodoyabashi → Midosuji → Namba</t>
         </is>
       </c>
       <c r="E82" s="25" t="n"/>
       <c r="F82" s="25" t="n"/>
       <c r="G82" s="25" t="inlineStr">
         <is>
-          <t>¥970, ~45min</t>
+          <t>¥430 + ¥240, ~1j15m. Sampai Namba ~16:45</t>
         </is>
       </c>
       <c r="H82" s="25" t="inlineStr">
@@ -3451,7 +3491,7 @@
         </is>
       </c>
       <c r="I82" s="26" t="n">
-        <v>970</v>
+        <v>670</v>
       </c>
       <c r="J82" s="26">
         <f>I82*'Budget Summary'!$B$2</f>
@@ -3459,91 +3499,104 @@
       </c>
     </row>
     <row r="83" ht="27.75" customHeight="1" s="23">
-      <c r="A83" s="27" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B83" s="27" t="inlineStr">
-        <is>
-          <t>12 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C83" s="27" t="inlineStr">
-        <is>
-          <t>~05:38</t>
-        </is>
-      </c>
-      <c r="D83" s="27" t="inlineStr">
-        <is>
-          <t>Subuh (kat guesthouse sblm gerak / atas train)</t>
-        </is>
-      </c>
-      <c r="E83" s="27" t="inlineStr">
-        <is>
-          <t>Subuh ~05:38</t>
-        </is>
-      </c>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
-      <c r="H83" s="27" t="n"/>
-      <c r="I83" s="28" t="n"/>
-      <c r="J83" s="28" t="n"/>
+      <c r="A83" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B83" s="25" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C83" s="25" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D83" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib</t>
+        </is>
+      </c>
+      <c r="E83" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib 17:00</t>
+        </is>
+      </c>
+      <c r="F83" s="25" t="n"/>
+      <c r="G83" s="25" t="n"/>
+      <c r="H83" s="25" t="n"/>
+      <c r="I83" s="26" t="n"/>
+      <c r="J83" s="26" t="n"/>
     </row>
     <row r="84" ht="27.75" customHeight="1" s="23">
-      <c r="A84" s="25" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B84" s="25" t="inlineStr">
-        <is>
-          <t>12 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C84" s="25" t="inlineStr">
-        <is>
-          <t>05:50</t>
-        </is>
-      </c>
-      <c r="D84" s="25" t="inlineStr">
-        <is>
-          <t>Sampai KIX — check-in, imigresen, security</t>
-        </is>
-      </c>
-      <c r="E84" s="25" t="n"/>
-      <c r="F84" s="25" t="n"/>
-      <c r="G84" s="25" t="inlineStr">
-        <is>
-          <t>Sampai ~2j sblm flight</t>
-        </is>
-      </c>
-      <c r="H84" s="25" t="n"/>
-      <c r="I84" s="26" t="n"/>
-      <c r="J84" s="26" t="n"/>
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D84" s="29" t="inlineStr">
+        <is>
+          <t>Dinner — masak (habiskan baki bahan)</t>
+        </is>
+      </c>
+      <c r="E84" s="29" t="n"/>
+      <c r="F84" s="29" t="inlineStr">
+        <is>
+          <t>Masak</t>
+        </is>
+      </c>
+      <c r="G84" s="29" t="n"/>
+      <c r="H84" s="29" t="inlineStr">
+        <is>
+          <t>Food-Masak</t>
+        </is>
+      </c>
+      <c r="I84" s="30" t="n">
+        <v>700</v>
+      </c>
+      <c r="J84" s="30">
+        <f>I84*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="85" ht="27.75" customHeight="1" s="23">
       <c r="A85" s="25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C85" s="25" t="inlineStr">
         <is>
-          <t>07:10</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D85" s="25" t="inlineStr">
         <is>
-          <t>Boarding</t>
-        </is>
-      </c>
-      <c r="E85" s="25" t="n"/>
+          <t>Isyak</t>
+        </is>
+      </c>
+      <c r="E85" s="25" t="inlineStr">
+        <is>
+          <t>Isyak 18:20</t>
+        </is>
+      </c>
       <c r="F85" s="25" t="n"/>
       <c r="G85" s="25" t="n"/>
       <c r="H85" s="25" t="n"/>
@@ -3553,22 +3606,22 @@
     <row r="86" ht="27.75" customHeight="1" s="23">
       <c r="A86" s="25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C86" s="25" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D86" s="25" t="inlineStr">
         <is>
-          <t>Take off — balik Incheon</t>
+          <t>Kemas beg, tidur awal (flight awal esok!)</t>
         </is>
       </c>
       <c r="E86" s="25" t="n"/>
@@ -3577,6 +3630,196 @@
       <c r="H86" s="25" t="n"/>
       <c r="I86" s="26" t="n"/>
       <c r="J86" s="26" t="n"/>
+    </row>
+    <row r="87" ht="27.75" customHeight="1" s="23">
+      <c r="A87" s="27" t="inlineStr">
+        <is>
+          <t>7
+(Selasa)</t>
+        </is>
+      </c>
+      <c r="B87" s="27" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C87" s="27" t="inlineStr">
+        <is>
+          <t>~04:30</t>
+        </is>
+      </c>
+      <c r="D87" s="27" t="inlineStr">
+        <is>
+          <t>Bangun awal</t>
+        </is>
+      </c>
+      <c r="E87" s="27" t="n"/>
+      <c r="F87" s="27" t="n"/>
+      <c r="G87" s="27" t="n"/>
+      <c r="H87" s="27" t="n"/>
+      <c r="I87" s="28" t="n"/>
+      <c r="J87" s="28" t="n"/>
+    </row>
+    <row r="88" ht="27.75" customHeight="1" s="23">
+      <c r="A88" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B88" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C88" s="25" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="D88" s="25" t="inlineStr">
+        <is>
+          <t>Nankai Airport Express Namba → KIX</t>
+        </is>
+      </c>
+      <c r="E88" s="25" t="n"/>
+      <c r="F88" s="25" t="n"/>
+      <c r="G88" s="25" t="inlineStr">
+        <is>
+          <t>¥970, ~45min</t>
+        </is>
+      </c>
+      <c r="H88" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I88" s="26" t="n">
+        <v>970</v>
+      </c>
+      <c r="J88" s="26">
+        <f>I88*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="27.75" customHeight="1" s="23">
+      <c r="A89" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B89" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C89" s="25" t="inlineStr">
+        <is>
+          <t>~05:38</t>
+        </is>
+      </c>
+      <c r="D89" s="25" t="inlineStr">
+        <is>
+          <t>Subuh (kat guesthouse sblm gerak / atas train)</t>
+        </is>
+      </c>
+      <c r="E89" s="25" t="inlineStr">
+        <is>
+          <t>Subuh ~05:38</t>
+        </is>
+      </c>
+      <c r="F89" s="25" t="n"/>
+      <c r="G89" s="25" t="n"/>
+      <c r="H89" s="25" t="n"/>
+      <c r="I89" s="26" t="n"/>
+      <c r="J89" s="26" t="n"/>
+    </row>
+    <row r="90" ht="27.75" customHeight="1" s="23">
+      <c r="A90" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B90" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C90" s="25" t="inlineStr">
+        <is>
+          <t>05:50</t>
+        </is>
+      </c>
+      <c r="D90" s="25" t="inlineStr">
+        <is>
+          <t>Sampai KIX — check-in, imigresen, security</t>
+        </is>
+      </c>
+      <c r="E90" s="25" t="n"/>
+      <c r="F90" s="25" t="n"/>
+      <c r="G90" s="25" t="inlineStr">
+        <is>
+          <t>Sampai ~2j sblm flight</t>
+        </is>
+      </c>
+      <c r="H90" s="25" t="n"/>
+      <c r="I90" s="26" t="n"/>
+      <c r="J90" s="26" t="n"/>
+    </row>
+    <row r="91" ht="27.75" customHeight="1" s="23">
+      <c r="A91" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B91" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C91" s="25" t="inlineStr">
+        <is>
+          <t>07:10</t>
+        </is>
+      </c>
+      <c r="D91" s="25" t="inlineStr">
+        <is>
+          <t>Boarding</t>
+        </is>
+      </c>
+      <c r="E91" s="25" t="n"/>
+      <c r="F91" s="25" t="n"/>
+      <c r="G91" s="25" t="n"/>
+      <c r="H91" s="25" t="n"/>
+      <c r="I91" s="26" t="n"/>
+      <c r="J91" s="26" t="n"/>
+    </row>
+    <row r="92" ht="27.75" customHeight="1" s="23">
+      <c r="A92" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B92" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C92" s="25" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="D92" s="25" t="inlineStr">
+        <is>
+          <t>Take off — balik Incheon</t>
+        </is>
+      </c>
+      <c r="E92" s="25" t="n"/>
+      <c r="F92" s="25" t="n"/>
+      <c r="G92" s="25" t="n"/>
+      <c r="H92" s="25" t="n"/>
+      <c r="I92" s="26" t="n"/>
+      <c r="J92" s="26" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3720,11 +3963,11 @@
     <row r="12" ht="15" customHeight="1" s="23">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>Transport (bas/train intercity + local)</t>
+          <t>Transport (bas malam + kereta sewa Fuji + train/metro)</t>
         </is>
       </c>
       <c r="B12" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E12,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E12,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C12" s="26">
@@ -3748,7 +3991,7 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E13,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E13,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C13" s="26">
@@ -3768,11 +4011,11 @@
     <row r="14" ht="15" customHeight="1" s="23">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>Penginapan tambahan (manga cafe Tokyo x2)</t>
+          <t>Penginapan tambahan (manga cafe Tokyo x1; malam Sabtu tidur dalam kereta)</t>
         </is>
       </c>
       <c r="B14" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E14,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E14,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C14" s="26">
@@ -3796,7 +4039,7 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E15,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E15,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C15" s="26">
@@ -3820,7 +4063,7 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E16,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E16,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C16" s="26">
@@ -3844,7 +4087,7 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E17,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E17,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C17" s="26">
@@ -3868,7 +4111,7 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$86,E18,Itinerary!$I$2:$I$86)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$92,E18,Itinerary!$I$2:$I$92)</f>
         <v/>
       </c>
       <c r="C18" s="26">
@@ -3947,7 +4190,7 @@
     <row r="26" ht="30" customHeight="1" s="23">
       <c r="A26" s="40" t="inlineStr">
         <is>
-          <t>Nota: Food-Bekal (Hari 5 lunch) dah termasuk dalam pembelian Hari 4 dinner. Kos masak = anggaran groceries sahaja, ANDAI guesthouse ada dapur — SAHKAN dengan host dulu.</t>
+          <t>Nota: Food-Bekal = snek malam + sarapan dalam kereta (Hari 4). Kereta sewa = anggaran Toyota W2 + tayar salji + insurans, SEMAK harga sebenar masa booking. Kos masak = anggaran groceries sahaja.</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4353,7 @@
     <row r="13" ht="45" customHeight="1" s="23">
       <c r="A13" s="43" t="inlineStr">
         <is>
-          <t>PENTING — Hari 3, 5, 6: Subuh mungkin jatuh time atas bas overnight. Sedia air sembahyang/tayammum kering, guna qiblat app, dan boleh jamak/qada bila sampai destinasi kalau betul-betul tak boleh solat atas bas.</t>
+          <t>PENTING — Hari 3 &amp; 6: Subuh jatuh time atas bas overnight. Sedia air sembahyang/tayammum kering, guna qiblat app, dan boleh jamak/qada bila sampai kalau betul-betul tak boleh solat atas bas. Hari 5: Subuh di tepi tasik Kawaguchiko (bawa sejadah).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch Tokyo nights to 9STAY apartment.
</commit_message>
<xml_diff>
--- a/Japan_Winter_Trip_Itinerary.xlsx
+++ b/Japan_Winter_Trip_Itinerary.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="22" min="1" max="1"/>
@@ -1625,14 +1625,14 @@
       </c>
       <c r="D31" s="25" t="inlineStr">
         <is>
-          <t>Sampai Tokyo (bus terminal Shinjuku)</t>
+          <t>Sampai Tokyo (Busta Shinjuku)</t>
         </is>
       </c>
       <c r="E31" s="25" t="n"/>
       <c r="F31" s="25" t="n"/>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>Freshen up kat terminal</t>
+          <t>Freshen up kat terminal. Bagasi masuk coin locker Busta Shinjuku sampai petang</t>
         </is>
       </c>
       <c r="H31" s="25" t="n"/>
@@ -1754,40 +1754,40 @@
       <c r="J34" s="26" t="n"/>
     </row>
     <row r="35" ht="27.75" customHeight="1" s="23">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B35" s="27" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
       </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C35" s="25" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="D35" s="27" t="inlineStr">
+      <c r="D35" s="25" t="inlineStr">
         <is>
           <t>SOLAT JUMAAT kat Tokyo Camii (lelaki sampai sebelum 12:15). Perempuan: ikut Jumaat di ruang wanita, atau Zohor biasa</t>
         </is>
       </c>
-      <c r="E35" s="27" t="inlineStr">
+      <c r="E35" s="25" t="inlineStr">
         <is>
           <t>Jumaat ~13:00 (azan ~12:30)</t>
         </is>
       </c>
-      <c r="F35" s="27" t="n"/>
-      <c r="G35" s="27" t="inlineStr">
+      <c r="F35" s="25" t="n"/>
+      <c r="G35" s="25" t="inlineStr">
         <is>
           <t>Khutbah dalam bahasa Jepun, Turki &amp; Inggeris</t>
         </is>
       </c>
-      <c r="H35" s="27" t="n"/>
-      <c r="I35" s="28" t="n"/>
-      <c r="J35" s="28" t="n"/>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="26" t="n"/>
+      <c r="J35" s="26" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="23">
       <c r="A36" s="25" t="inlineStr">
@@ -1831,36 +1831,36 @@
       </c>
     </row>
     <row r="37" ht="27.75" customHeight="1" s="23">
-      <c r="A37" s="27" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B37" s="27" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
       </c>
-      <c r="C37" s="27" t="inlineStr">
+      <c r="C37" s="25" t="inlineStr">
         <is>
           <t>14:20</t>
         </is>
       </c>
-      <c r="D37" s="27" t="inlineStr">
-        <is>
-          <t>Asar</t>
-        </is>
-      </c>
-      <c r="E37" s="27" t="inlineStr">
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Asar (Tokyo Camii)</t>
+        </is>
+      </c>
+      <c r="E37" s="25" t="inlineStr">
         <is>
           <t>Asar 14:20</t>
         </is>
       </c>
-      <c r="F37" s="27" t="n"/>
-      <c r="G37" s="27" t="n"/>
-      <c r="H37" s="27" t="n"/>
-      <c r="I37" s="28" t="n"/>
-      <c r="J37" s="28" t="n"/>
+      <c r="F37" s="25" t="n"/>
+      <c r="G37" s="25" t="n"/>
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="26" t="n"/>
     </row>
     <row r="38" ht="27.75" customHeight="1" s="23">
       <c r="A38" s="25" t="inlineStr">
@@ -1875,52 +1875,60 @@
       </c>
       <c r="C38" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D38" s="25" t="inlineStr">
         <is>
-          <t>Shibuya / Harajuku</t>
+          <t>Ambil bagasi Busta Shinjuku → JR Yamanote ke Otsuka (~10min)</t>
         </is>
       </c>
       <c r="E38" s="25" t="n"/>
       <c r="F38" s="25" t="n"/>
-      <c r="G38" s="25" t="n"/>
+      <c r="G38" s="25" t="inlineStr">
+        <is>
+          <t>Atau Marunouchi Line ke Shin-otsuka (330m dari apartment)</t>
+        </is>
+      </c>
       <c r="H38" s="25" t="n"/>
       <c r="I38" s="26" t="n"/>
       <c r="J38" s="26" t="n"/>
     </row>
     <row r="39" ht="27.75" customHeight="1" s="23">
-      <c r="A39" s="27" t="inlineStr">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B39" s="27" t="inlineStr">
+      <c r="B39" s="31" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
       </c>
-      <c r="C39" s="27" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="D39" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib</t>
-        </is>
-      </c>
-      <c r="E39" s="27" t="inlineStr">
-        <is>
-          <t>Maghrib 16:45</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="27" t="n"/>
-      <c r="H39" s="27" t="n"/>
-      <c r="I39" s="28" t="n"/>
-      <c r="J39" s="28" t="n"/>
+      <c r="C39" s="31" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>CHECK-IN 9STAY Bunkyo Otsuka (self check-in) — 2 malam, DAH BAYAR ✓</t>
+        </is>
+      </c>
+      <c r="E39" s="31" t="n"/>
+      <c r="F39" s="31" t="n"/>
+      <c r="G39" s="31" t="inlineStr">
+        <is>
+          <t>Check-in lepas 15:00, check-out sebelum 10:00 Ahad. Mandi &amp; rehat lepas bas malam</t>
+        </is>
+      </c>
+      <c r="H39" s="31" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="I39" s="32" t="n"/>
+      <c r="J39" s="32" t="n"/>
     </row>
     <row r="40" ht="27.75" customHeight="1" s="23">
       <c r="A40" s="25" t="inlineStr">
@@ -1935,65 +1943,52 @@
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="D40" s="25" t="inlineStr">
         <is>
-          <t>Dinner — halal Shinjuku area</t>
-        </is>
-      </c>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
+          <t>Maghrib (apartment)</t>
+        </is>
+      </c>
+      <c r="E40" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib 16:45</t>
+        </is>
+      </c>
+      <c r="F40" s="25" t="n"/>
       <c r="G40" s="25" t="n"/>
-      <c r="H40" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I40" s="26" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J40" s="26">
-        <f>I40*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="26" t="n"/>
+      <c r="J40" s="26" t="n"/>
     </row>
     <row r="41" ht="27.75" customHeight="1" s="23">
-      <c r="A41" s="27" t="inlineStr">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B41" s="27" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
       </c>
-      <c r="C41" s="27" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="D41" s="27" t="inlineStr">
-        <is>
-          <t>Isyak</t>
-        </is>
-      </c>
-      <c r="E41" s="27" t="inlineStr">
-        <is>
-          <t>Isyak 18:05</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="27" t="n"/>
-      <c r="I41" s="28" t="n"/>
-      <c r="J41" s="28" t="n"/>
+      <c r="C41" s="25" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="inlineStr">
+        <is>
+          <t>Shibuya Crossing &amp; Hachiko + Harajuku (malam, lampu dah menyala)</t>
+        </is>
+      </c>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="26" t="n"/>
+      <c r="J41" s="26" t="n"/>
     </row>
     <row r="42" ht="27.75" customHeight="1" s="23">
       <c r="A42" s="25" t="inlineStr">
@@ -2008,177 +2003,164 @@
       </c>
       <c r="C42" s="25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="D42" s="25" t="inlineStr">
         <is>
-          <t>Check-in manga cafe (private booth)</t>
-        </is>
-      </c>
-      <c r="E42" s="25" t="n"/>
+          <t>Isyak — surau Shibuya PARCO 5F</t>
+        </is>
+      </c>
+      <c r="E42" s="25" t="inlineStr">
+        <is>
+          <t>Isyak 18:05</t>
+        </is>
+      </c>
       <c r="F42" s="25" t="n"/>
-      <c r="G42" s="25" t="inlineStr">
-        <is>
-          <t>¥1,700-3,500/malam</t>
-        </is>
-      </c>
-      <c r="H42" s="25" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="I42" s="26" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J42" s="26">
-        <f>I42*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="G42" s="25" t="n"/>
+      <c r="H42" s="25" t="n"/>
+      <c r="I42" s="26" t="n"/>
+      <c r="J42" s="26" t="n"/>
     </row>
     <row r="43" ht="27.75" customHeight="1" s="23">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>8 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C43" s="25" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="inlineStr">
+        <is>
+          <t>Dinner — halal Shibuya/Shinjuku</t>
+        </is>
+      </c>
+      <c r="E43" s="25" t="n"/>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G43" s="25" t="n"/>
+      <c r="H43" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I43" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J43" s="26">
+        <f>I43*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="27.75" customHeight="1" s="23">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>8 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D44" s="25" t="inlineStr">
+        <is>
+          <t>Balik apartment, tidur awal (esok drive ke Fuji)</t>
+        </is>
+      </c>
+      <c r="E44" s="25" t="n"/>
+      <c r="F44" s="25" t="n"/>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="25" t="n"/>
+      <c r="I44" s="26" t="n"/>
+      <c r="J44" s="26" t="n"/>
+    </row>
+    <row r="45" ht="27.75" customHeight="1" s="23">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t>4
 (Sabtu)</t>
         </is>
       </c>
-      <c r="B43" s="27" t="inlineStr">
+      <c r="B45" s="27" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C43" s="27" t="inlineStr">
+      <c r="C45" s="27" t="inlineStr">
         <is>
           <t>05:22</t>
         </is>
       </c>
-      <c r="D43" s="27" t="inlineStr">
-        <is>
-          <t>Subuh (manga cafe / musolla berdekatan)</t>
-        </is>
-      </c>
-      <c r="E43" s="27" t="inlineStr">
+      <c r="D45" s="27" t="inlineStr">
+        <is>
+          <t>Subuh (apartment)</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr">
         <is>
           <t>Subuh 05:22</t>
         </is>
       </c>
-      <c r="F43" s="27" t="n"/>
-      <c r="G43" s="27" t="n"/>
-      <c r="H43" s="27" t="n"/>
-      <c r="I43" s="28" t="n"/>
-      <c r="J43" s="28" t="n"/>
-    </row>
-    <row r="44" ht="27.75" customHeight="1" s="23">
-      <c r="A44" s="25" t="inlineStr">
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+      <c r="H45" s="27" t="n"/>
+      <c r="I45" s="28" t="n"/>
+      <c r="J45" s="28" t="n"/>
+    </row>
+    <row r="46" ht="27.75" customHeight="1" s="23">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B44" s="25" t="inlineStr">
+      <c r="B46" s="25" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C44" s="25" t="inlineStr">
+      <c r="C46" s="25" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D44" s="25" t="inlineStr">
-        <is>
-          <t>Breakfast — conbini halal-safe (onigiri salmon/tuna)</t>
-        </is>
-      </c>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="25" t="inlineStr">
+      <c r="D46" s="25" t="inlineStr">
+        <is>
+          <t>Breakfast — conbini / masak kat apartment (kalau ada dapur)</t>
+        </is>
+      </c>
+      <c r="E46" s="25" t="n"/>
+      <c r="F46" s="25" t="inlineStr">
         <is>
           <t>Makan luar (halal)</t>
         </is>
       </c>
-      <c r="G44" s="25" t="n"/>
-      <c r="H44" s="25" t="inlineStr">
+      <c r="G46" s="25" t="n"/>
+      <c r="H46" s="25" t="inlineStr">
         <is>
           <t>Food-Luar</t>
         </is>
       </c>
-      <c r="I44" s="26" t="n">
+      <c r="I46" s="26" t="n">
         <v>600</v>
       </c>
-      <c r="J44" s="26">
-        <f>I44*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="27.75" customHeight="1" s="23">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="inlineStr">
-        <is>
-          <t>9 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C45" s="25" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="D45" s="25" t="inlineStr">
-        <is>
-          <t>Check-out manga cafe, bawa SEMUA bagasi ke Toyota Rent a Car Shinjuku</t>
-        </is>
-      </c>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="25" t="n"/>
-      <c r="G45" s="25" t="inlineStr">
-        <is>
-          <t>Beli kairo (heat pack) + air kat konbini untuk malam ni</t>
-        </is>
-      </c>
-      <c r="H45" s="25" t="n"/>
-      <c r="I45" s="26" t="n"/>
-      <c r="J45" s="26" t="n"/>
-    </row>
-    <row r="46" ht="27.75" customHeight="1" s="23">
-      <c r="A46" s="31" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B46" s="31" t="inlineStr">
-        <is>
-          <t>9 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C46" s="31" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="D46" s="31" t="inlineStr">
-        <is>
-          <t>AMBIL KERETA — Toyota Noah/Voxy (kelas W2, 7-8 seat) + tayar salji + kad ETC</t>
-        </is>
-      </c>
-      <c r="E46" s="31" t="n"/>
-      <c r="F46" s="31" t="n"/>
-      <c r="G46" s="31" t="inlineStr">
-        <is>
-          <t>WAJIB: passport + lesen Malaysia + IDP (buku fizikal) untuk 3 pemandu. Sewa ~¥37-45k + tayar salji ¥3,300/24j + insurans ≈ ¥52k ÷ 6</t>
-        </is>
-      </c>
-      <c r="H46" s="31" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I46" s="32" t="n">
-        <v>8700</v>
-      </c>
-      <c r="J46" s="32">
+      <c r="J46" s="26">
         <f>I46*'Budget Summary'!$B$2</f>
         <v/>
       </c>
@@ -2196,65 +2178,65 @@
       </c>
       <c r="C47" s="25" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="D47" s="25" t="inlineStr">
         <is>
-          <t>Drive Shinjuku → Kawaguchiko (Chuo Expressway → Kawaguchiko IC)</t>
+          <t>JR Otsuka → Shinjuku (~10min), jalan ke Toyota Rent a Car Shinjuku</t>
         </is>
       </c>
       <c r="E47" s="25" t="n"/>
       <c r="F47" s="25" t="n"/>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>Tol ETC ~¥2,600 ÷ 6. ~1j30m kalau lancar — cuti panjang 3 hari, jangka 2j+</t>
-        </is>
-      </c>
-      <c r="H47" s="25" t="inlineStr">
+          <t>Beli air + snek untuk perjalanan</t>
+        </is>
+      </c>
+      <c r="H47" s="25" t="n"/>
+      <c r="I47" s="26" t="n"/>
+      <c r="J47" s="26" t="n"/>
+    </row>
+    <row r="48" ht="27.75" customHeight="1" s="23">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C48" s="31" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>AMBIL KERETA — Toyota Noah/Voxy (kelas W2, 7-8 seat) + tayar salji + kad ETC</t>
+        </is>
+      </c>
+      <c r="E48" s="31" t="n"/>
+      <c r="F48" s="31" t="n"/>
+      <c r="G48" s="31" t="inlineStr">
+        <is>
+          <t>WAJIB: passport + lesen Malaysia + IDP (buku fizikal) untuk 3 pemandu. Sewa Sab 08:00 → Ahd ~10:30 (~26j) ≈ ¥35k + tayar salji ¥6,600 + insurans ≈ ¥46k ÷ 6</t>
+        </is>
+      </c>
+      <c r="H48" s="31" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="I47" s="26" t="n">
-        <v>450</v>
-      </c>
-      <c r="J47" s="26">
-        <f>I47*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="27.75" customHeight="1" s="23">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="inlineStr">
-        <is>
-          <t>9 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C48" s="25" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="inlineStr">
-        <is>
-          <t>Chureito Pagoda — 398 anak tangga, Fuji paling jelas waktu pagi</t>
-        </is>
-      </c>
-      <c r="E48" s="25" t="n"/>
-      <c r="F48" s="25" t="n"/>
-      <c r="G48" s="25" t="inlineStr">
-        <is>
-          <t>Parking Arakurayama Sengen Park (cepat penuh hujung minggu). Tangga mungkin berais</t>
-        </is>
-      </c>
-      <c r="H48" s="25" t="n"/>
-      <c r="I48" s="26" t="n"/>
-      <c r="J48" s="26" t="n"/>
+      <c r="I48" s="32" t="n">
+        <v>7700</v>
+      </c>
+      <c r="J48" s="32">
+        <f>I48*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="27.75" customHeight="1" s="23">
       <c r="A49" s="25" t="inlineStr">
@@ -2269,32 +2251,28 @@
       </c>
       <c r="C49" s="25" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="D49" s="25" t="inlineStr">
         <is>
-          <t>Lunch — T&amp;T Fujiyama Halal Restaurant (hoto halal, mi tradisional Yamanashi)</t>
+          <t>Drive Shinjuku → Kawaguchiko (Chuo Expressway → Kawaguchiko IC)</t>
         </is>
       </c>
       <c r="E49" s="25" t="n"/>
-      <c r="F49" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
+      <c r="F49" s="25" t="n"/>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>Fujiyoshida, ~10min drive dari Chureito. Semua hoto ¥1,000. Buka 11:30-19:30</t>
+          <t>Tol ETC ~¥2,600 ÷ 6. ~1j30m kalau lancar — cuti panjang 3 hari, jangka 2j+</t>
         </is>
       </c>
       <c r="H49" s="25" t="inlineStr">
         <is>
-          <t>Food-Luar</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="I49" s="26" t="n">
-        <v>1000</v>
+        <v>450</v>
       </c>
       <c r="J49" s="26">
         <f>I49*'Budget Summary'!$B$2</f>
@@ -2314,23 +2292,19 @@
       </c>
       <c r="C50" s="25" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>Zohor — Masjid Fujikawaguchiko (Funatsu, dekat stesen Kawaguchiko)</t>
-        </is>
-      </c>
-      <c r="E50" s="25" t="inlineStr">
-        <is>
-          <t>Zohor (masuk ~11:50)</t>
-        </is>
-      </c>
+          <t>Chureito Pagoda — 398 anak tangga, Fuji paling jelas waktu pagi</t>
+        </is>
+      </c>
+      <c r="E50" s="25" t="n"/>
       <c r="F50" s="25" t="n"/>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>Masjid dibuka 2020, ada kafe halal dalam bangunan sama</t>
+          <t>Parking Arakurayama Sengen Park (cepat penuh hujung minggu). Tangga mungkin berais</t>
         </is>
       </c>
       <c r="H50" s="25" t="n"/>
@@ -2350,20 +2324,37 @@
       </c>
       <c r="C51" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D51" s="25" t="inlineStr">
         <is>
-          <t>Oishi Park — view Fuji dari seberang tasik Kawaguchiko (percuma)</t>
+          <t>Lunch — T&amp;T Fujiyama Halal Restaurant (hoto halal, mi tradisional Yamanashi)</t>
         </is>
       </c>
       <c r="E51" s="25" t="n"/>
-      <c r="F51" s="25" t="n"/>
-      <c r="G51" s="25" t="n"/>
-      <c r="H51" s="25" t="n"/>
-      <c r="I51" s="26" t="n"/>
-      <c r="J51" s="26" t="n"/>
+      <c r="F51" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G51" s="25" t="inlineStr">
+        <is>
+          <t>Fujiyoshida, ~10min drive dari Chureito. Semua hoto ¥1,000. Buka 11:30-19:30</t>
+        </is>
+      </c>
+      <c r="H51" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I51" s="26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J51" s="26">
+        <f>I51*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="27.75" customHeight="1" s="23">
       <c r="A52" s="25" t="inlineStr">
@@ -2378,21 +2369,25 @@
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D52" s="25" t="inlineStr">
         <is>
-          <t>Asar</t>
+          <t>Zohor — Masjid Fujikawaguchiko (Funatsu, dekat stesen Kawaguchiko)</t>
         </is>
       </c>
       <c r="E52" s="25" t="inlineStr">
         <is>
-          <t>Asar ~14:15</t>
+          <t>Zohor (masuk ~11:50)</t>
         </is>
       </c>
       <c r="F52" s="25" t="n"/>
-      <c r="G52" s="25" t="n"/>
+      <c r="G52" s="25" t="inlineStr">
+        <is>
+          <t>Masjid dibuka 2020, ada kafe halal dalam bangunan sama</t>
+        </is>
+      </c>
       <c r="H52" s="25" t="n"/>
       <c r="I52" s="26" t="n"/>
       <c r="J52" s="26" t="n"/>
@@ -2410,21 +2405,17 @@
       </c>
       <c r="C53" s="25" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D53" s="25" t="inlineStr">
         <is>
-          <t>Oshino Hakkai — 8 kolam air mata air Fuji (percuma), ~25min drive</t>
+          <t>Oishi Park — view Fuji dari seberang tasik Kawaguchiko (percuma)</t>
         </is>
       </c>
       <c r="E53" s="25" t="n"/>
       <c r="F53" s="25" t="n"/>
-      <c r="G53" s="25" t="inlineStr">
-        <is>
-          <t>Air salji Fuji ditapis lava berpuluh tahun — boleh isi botol &amp; minum</t>
-        </is>
-      </c>
+      <c r="G53" s="25" t="n"/>
       <c r="H53" s="25" t="n"/>
       <c r="I53" s="26" t="n"/>
       <c r="J53" s="26" t="n"/>
@@ -2442,17 +2433,17 @@
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="D54" s="25" t="inlineStr">
         <is>
-          <t>Maghrib — Masjid Fujikawaguchiko</t>
+          <t>Asar</t>
         </is>
       </c>
       <c r="E54" s="25" t="inlineStr">
         <is>
-          <t>Maghrib ~16:45</t>
+          <t>Asar ~14:15</t>
         </is>
       </c>
       <c r="F54" s="25" t="n"/>
@@ -2474,33 +2465,24 @@
       </c>
       <c r="C55" s="25" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D55" s="25" t="inlineStr">
         <is>
-          <t>Dinner — Halal food and cafe (Masjid) / Idaten Bettei (halal, dekat stesen)</t>
+          <t>Oshino Hakkai — 8 kolam air mata air Fuji (percuma), ~25min drive</t>
         </is>
       </c>
       <c r="E55" s="25" t="n"/>
-      <c r="F55" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
-      <c r="G55" s="25" t="n"/>
-      <c r="H55" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I55" s="26" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J55" s="26">
-        <f>I55*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="F55" s="25" t="n"/>
+      <c r="G55" s="25" t="inlineStr">
+        <is>
+          <t>Air salji Fuji ditapis lava berpuluh tahun — boleh isi botol &amp; minum</t>
+        </is>
+      </c>
+      <c r="H55" s="25" t="n"/>
+      <c r="I55" s="26" t="n"/>
+      <c r="J55" s="26" t="n"/>
     </row>
     <row r="56" ht="27.75" customHeight="1" s="23">
       <c r="A56" s="25" t="inlineStr">
@@ -2515,17 +2497,17 @@
       </c>
       <c r="C56" s="25" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="D56" s="25" t="inlineStr">
         <is>
-          <t>Isyak — Masjid Fujikawaguchiko</t>
+          <t>Maghrib — Masjid Fujikawaguchiko (sunset atas Fuji)</t>
         </is>
       </c>
       <c r="E56" s="25" t="inlineStr">
         <is>
-          <t>Isyak ~18:00</t>
+          <t>Maghrib ~16:45</t>
         </is>
       </c>
       <c r="F56" s="25" t="n"/>
@@ -2547,28 +2529,28 @@
       </c>
       <c r="C57" s="25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="D57" s="25" t="inlineStr">
         <is>
-          <t>Isi minyak + konbini: snek malam, sarapan esok, kairo, air</t>
+          <t>Dinner — Halal food and cafe (Masjid) / Idaten Bettei (halal, dekat stesen)</t>
         </is>
       </c>
       <c r="E57" s="25" t="n"/>
       <c r="F57" s="25" t="inlineStr">
         <is>
-          <t>Snek/Bekal</t>
+          <t>Makan luar (halal)</t>
         </is>
       </c>
       <c r="G57" s="25" t="n"/>
       <c r="H57" s="25" t="inlineStr">
         <is>
-          <t>Food-Bekal</t>
+          <t>Food-Luar</t>
         </is>
       </c>
       <c r="I57" s="26" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="J57" s="26">
         <f>I57*'Budget Summary'!$B$2</f>
@@ -2576,301 +2558,284 @@
       </c>
     </row>
     <row r="58" ht="27.75" customHeight="1" s="23">
-      <c r="A58" s="31" t="inlineStr">
+      <c r="A58" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B58" s="31" t="inlineStr">
+      <c r="B58" s="25" t="inlineStr">
         <is>
           <t>9 Jan 2027</t>
         </is>
       </c>
-      <c r="C58" s="31" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D58" s="31" t="inlineStr">
-        <is>
-          <t>TIDUR DALAM KERETA — Michi-no-eki Katsuyama (tepi tasik, parking percuma, tandas 24j)</t>
-        </is>
-      </c>
-      <c r="E58" s="31" t="n"/>
-      <c r="F58" s="31" t="n"/>
-      <c r="G58" s="31" t="inlineStr">
-        <is>
-          <t>SUHU purata −7°C (boleh −10°C). Enjin MATI masa semua tidur; salji boleh tutup ekzos → karbon monoksida. Sleeping bag −10°C + kairo + CO detector. JANGAN guna dapur gas</t>
-        </is>
-      </c>
-      <c r="H58" s="31" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="I58" s="32" t="n"/>
-      <c r="J58" s="32" t="n"/>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D58" s="25" t="inlineStr">
+        <is>
+          <t>Isyak — Masjid Fujikawaguchiko</t>
+        </is>
+      </c>
+      <c r="E58" s="25" t="inlineStr">
+        <is>
+          <t>Isyak ~18:00</t>
+        </is>
+      </c>
+      <c r="F58" s="25" t="n"/>
+      <c r="G58" s="25" t="n"/>
+      <c r="H58" s="25" t="n"/>
+      <c r="I58" s="26" t="n"/>
+      <c r="J58" s="26" t="n"/>
     </row>
     <row r="59" ht="27.75" customHeight="1" s="23">
-      <c r="A59" s="27" t="inlineStr">
+      <c r="A59" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B59" s="31" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C59" s="31" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D59" s="31" t="inlineStr">
+        <is>
+          <t>Drive balik Kawaguchiko → Tokyo (Chuo Expressway)</t>
+        </is>
+      </c>
+      <c r="E59" s="31" t="n"/>
+      <c r="F59" s="31" t="n"/>
+      <c r="G59" s="31" t="inlineStr">
+        <is>
+          <t>Tol ETC ~¥2,600 ÷ 6. ~1j45m-2j30m. MALAM + jalan mungkin berais: tukar pemandu setiap ~1j, rehat kat Dangozaka SA kalau mengantuk</t>
+        </is>
+      </c>
+      <c r="H59" s="31" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I59" s="32" t="n">
+        <v>450</v>
+      </c>
+      <c r="J59" s="32">
+        <f>I59*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="27.75" customHeight="1" s="23">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B60" s="31" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C60" s="31" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D60" s="31" t="inlineStr">
+        <is>
+          <t>Isi minyak + parking semalaman dekat apartment (coin parking / akippa)</t>
+        </is>
+      </c>
+      <c r="E60" s="31" t="n"/>
+      <c r="F60" s="31" t="n"/>
+      <c r="G60" s="31" t="inlineStr">
+        <is>
+          <t>Minyak ~¥5k + parking Fuji ~¥1k + parking Tokyo semalam ~¥2-3k ÷ 6. Book parking awal — apartment takde parking</t>
+        </is>
+      </c>
+      <c r="H60" s="31" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I60" s="32" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J60" s="32">
+        <f>I60*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="27.75" customHeight="1" s="23">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B61" s="25" t="inlineStr">
+        <is>
+          <t>9 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C61" s="25" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="25" t="inlineStr">
+        <is>
+          <t>Tidur (apartment)</t>
+        </is>
+      </c>
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="25" t="n"/>
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="25" t="n"/>
+      <c r="I61" s="26" t="n"/>
+      <c r="J61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="27.75" customHeight="1" s="23">
+      <c r="A62" s="27" t="inlineStr">
         <is>
           <t>5
 (Ahad)</t>
         </is>
       </c>
-      <c r="B59" s="27" t="inlineStr">
+      <c r="B62" s="27" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C59" s="27" t="inlineStr">
+      <c r="C62" s="27" t="inlineStr">
         <is>
           <t>05:22</t>
         </is>
       </c>
-      <c r="D59" s="27" t="inlineStr">
-        <is>
-          <t>Subuh (Michi-no-eki / tepi tasik — bawa sejadah)</t>
-        </is>
-      </c>
-      <c r="E59" s="27" t="inlineStr">
-        <is>
-          <t>Subuh ~05:22</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="27" t="n"/>
-      <c r="H59" s="27" t="n"/>
-      <c r="I59" s="28" t="n"/>
-      <c r="J59" s="28" t="n"/>
-    </row>
-    <row r="60" ht="27.75" customHeight="1" s="23">
-      <c r="A60" s="25" t="inlineStr">
+      <c r="D62" s="27" t="inlineStr">
+        <is>
+          <t>Subuh (apartment)</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
+        <is>
+          <t>Subuh 05:22</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="n"/>
+      <c r="G62" s="27" t="n"/>
+      <c r="H62" s="27" t="n"/>
+      <c r="I62" s="28" t="n"/>
+      <c r="J62" s="28" t="n"/>
+    </row>
+    <row r="63" ht="27.75" customHeight="1" s="23">
+      <c r="A63" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B60" s="25" t="inlineStr">
+      <c r="B63" s="25" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C60" s="25" t="inlineStr">
-        <is>
-          <t>06:30</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="inlineStr">
-        <is>
-          <t>Matahari terbit + Fuji — Oishi Park / tepi tasik (~06:50)</t>
-        </is>
-      </c>
-      <c r="E60" s="25" t="n"/>
-      <c r="F60" s="25" t="n"/>
-      <c r="G60" s="25" t="inlineStr">
-        <is>
-          <t>Pagi = Fuji paling jelas, tasik paling tenang</t>
-        </is>
-      </c>
-      <c r="H60" s="25" t="n"/>
-      <c r="I60" s="26" t="n"/>
-      <c r="J60" s="26" t="n"/>
-    </row>
-    <row r="61" ht="27.75" customHeight="1" s="23">
-      <c r="A61" s="25" t="inlineStr">
+      <c r="C63" s="25" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="inlineStr">
+        <is>
+          <t>Breakfast — conbini / masak kat apartment</t>
+        </is>
+      </c>
+      <c r="E63" s="25" t="n"/>
+      <c r="F63" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G63" s="25" t="n"/>
+      <c r="H63" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I63" s="26" t="n">
+        <v>600</v>
+      </c>
+      <c r="J63" s="26">
+        <f>I63*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="27.75" customHeight="1" s="23">
+      <c r="A64" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B61" s="25" t="inlineStr">
+      <c r="B64" s="31" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C61" s="25" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="D61" s="25" t="inlineStr">
-        <is>
-          <t>Breakfast — snek/konbini</t>
-        </is>
-      </c>
-      <c r="E61" s="25" t="n"/>
-      <c r="F61" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
-      <c r="G61" s="25" t="n"/>
-      <c r="H61" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I61" s="26" t="n">
-        <v>600</v>
-      </c>
-      <c r="J61" s="26">
-        <f>I61*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="27.75" customHeight="1" s="23">
-      <c r="A62" s="25" t="inlineStr">
+      <c r="C64" s="31" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D64" s="31" t="inlineStr">
+        <is>
+          <t>Kemas &amp; CHECK-OUT sebelum 10:00 — semua bagasi masuk kereta</t>
+        </is>
+      </c>
+      <c r="E64" s="31" t="n"/>
+      <c r="F64" s="31" t="n"/>
+      <c r="G64" s="31" t="inlineStr">
+        <is>
+          <t>Check-out paling lewat 10:00</t>
+        </is>
+      </c>
+      <c r="H64" s="31" t="n"/>
+      <c r="I64" s="32" t="n"/>
+      <c r="J64" s="32" t="n"/>
+    </row>
+    <row r="65" ht="27.75" customHeight="1" s="23">
+      <c r="A65" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B62" s="25" t="inlineStr">
+      <c r="B65" s="31" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C62" s="25" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="D62" s="25" t="inlineStr">
-        <is>
-          <t>Drive balik Kawaguchiko → Shinjuku</t>
-        </is>
-      </c>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="25" t="n"/>
-      <c r="G62" s="25" t="inlineStr">
-        <is>
-          <t>Tol ETC ~¥2,600 ÷ 6. Ahad pagi arah Tokyo biasanya lancar (orang balik Isnin)</t>
-        </is>
-      </c>
-      <c r="H62" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I62" s="26" t="n">
-        <v>450</v>
-      </c>
-      <c r="J62" s="26">
-        <f>I62*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="27.75" customHeight="1" s="23">
-      <c r="A63" s="31" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B63" s="31" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C63" s="31" t="inlineStr">
-        <is>
-          <t>10:45</t>
-        </is>
-      </c>
-      <c r="D63" s="31" t="inlineStr">
-        <is>
-          <t>Isi minyak penuh &amp; PULANGKAN KERETA (Shinjuku)</t>
-        </is>
-      </c>
-      <c r="E63" s="31" t="n"/>
-      <c r="F63" s="31" t="n"/>
-      <c r="G63" s="31" t="inlineStr">
-        <is>
-          <t>Minyak ~¥5k + parking ~¥1k ÷ 6. Lewat pulang = caj ~¥2,860/jam. Bagasi masuk coin locker Busta Shinjuku</t>
-        </is>
-      </c>
-      <c r="H63" s="31" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I63" s="32" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J63" s="32">
-        <f>I63*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="27.75" customHeight="1" s="23">
-      <c r="A64" s="25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B64" s="25" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C64" s="25" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="D64" s="25" t="inlineStr">
-        <is>
-          <t>Local transport Tokyo (metro/IC card)</t>
-        </is>
-      </c>
-      <c r="E64" s="25" t="n"/>
-      <c r="F64" s="25" t="n"/>
-      <c r="G64" s="25" t="inlineStr">
-        <is>
-          <t>~¥800/hari</t>
-        </is>
-      </c>
-      <c r="H64" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I64" s="26" t="n">
-        <v>800</v>
-      </c>
-      <c r="J64" s="26">
-        <f>I64*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="27.75" customHeight="1" s="23">
-      <c r="A65" s="25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B65" s="25" t="inlineStr">
-        <is>
-          <t>10 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C65" s="25" t="inlineStr">
-        <is>
-          <t>11:47</t>
-        </is>
-      </c>
-      <c r="D65" s="25" t="inlineStr">
-        <is>
-          <t>Zohor</t>
-        </is>
-      </c>
-      <c r="E65" s="25" t="inlineStr">
-        <is>
-          <t>Zohor 11:47</t>
-        </is>
-      </c>
-      <c r="F65" s="25" t="n"/>
-      <c r="G65" s="25" t="n"/>
-      <c r="H65" s="25" t="n"/>
-      <c r="I65" s="26" t="n"/>
-      <c r="J65" s="26" t="n"/>
+      <c r="C65" s="31" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D65" s="31" t="inlineStr">
+        <is>
+          <t>Drive ke Shinjuku, isi minyak penuh, PULANGKAN KERETA (~10:30)</t>
+        </is>
+      </c>
+      <c r="E65" s="31" t="n"/>
+      <c r="F65" s="31" t="n"/>
+      <c r="G65" s="31" t="inlineStr">
+        <is>
+          <t>Lewat pulang = caj ~¥2,860/jam. Bagasi masuk coin locker Busta Shinjuku</t>
+        </is>
+      </c>
+      <c r="H65" s="31" t="n"/>
+      <c r="I65" s="32" t="n"/>
+      <c r="J65" s="32" t="n"/>
     </row>
     <row r="66" ht="27.75" customHeight="1" s="23">
       <c r="A66" s="25" t="inlineStr">
@@ -2885,28 +2850,28 @@
       </c>
       <c r="C66" s="25" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="D66" s="25" t="inlineStr">
         <is>
-          <t>Lunch — halal (Shinjuku/Shibuya)</t>
+          <t>Local transport Tokyo (metro/IC card)</t>
         </is>
       </c>
       <c r="E66" s="25" t="n"/>
-      <c r="F66" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
-      <c r="G66" s="25" t="n"/>
+      <c r="F66" s="25" t="n"/>
+      <c r="G66" s="25" t="inlineStr">
+        <is>
+          <t>~¥800/hari</t>
+        </is>
+      </c>
       <c r="H66" s="25" t="inlineStr">
         <is>
-          <t>Food-Luar</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="I66" s="26" t="n">
-        <v>1800</v>
+        <v>800</v>
       </c>
       <c r="J66" s="26">
         <f>I66*'Budget Summary'!$B$2</f>
@@ -2926,19 +2891,15 @@
       </c>
       <c r="C67" s="25" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="D67" s="25" t="inlineStr">
         <is>
-          <t>Asar</t>
-        </is>
-      </c>
-      <c r="E67" s="25" t="inlineStr">
-        <is>
-          <t>Asar 14:20</t>
-        </is>
-      </c>
+          <t>Akihabara (anime, game, arcade)</t>
+        </is>
+      </c>
+      <c r="E67" s="25" t="n"/>
       <c r="F67" s="25" t="n"/>
       <c r="G67" s="25" t="n"/>
       <c r="H67" s="25" t="n"/>
@@ -2958,33 +2919,24 @@
       </c>
       <c r="C68" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>11:47</t>
         </is>
       </c>
       <c r="D68" s="25" t="inlineStr">
         <is>
-          <t>Shibuya Sky — slot 14:30 (OPTIONAL, boleh skip)</t>
-        </is>
-      </c>
-      <c r="E68" s="25" t="n"/>
+          <t>Zohor — Masjid Nusantara, Akihabara</t>
+        </is>
+      </c>
+      <c r="E68" s="25" t="inlineStr">
+        <is>
+          <t>Zohor 11:47</t>
+        </is>
+      </c>
       <c r="F68" s="25" t="n"/>
-      <c r="G68" s="25" t="inlineStr">
-        <is>
-          <t>¥2,700 online. Tiket untuk Ahad 10 Jan buka 27 Dis 00:00. Keluar sebelum Maghrib ~16:45</t>
-        </is>
-      </c>
-      <c r="H68" s="25" t="inlineStr">
-        <is>
-          <t>Attraction-Optional</t>
-        </is>
-      </c>
-      <c r="I68" s="26" t="n">
-        <v>2700</v>
-      </c>
-      <c r="J68" s="26">
-        <f>I68*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="G68" s="25" t="n"/>
+      <c r="H68" s="25" t="n"/>
+      <c r="I68" s="26" t="n"/>
+      <c r="J68" s="26" t="n"/>
     </row>
     <row r="69" ht="27.75" customHeight="1" s="23">
       <c r="A69" s="25" t="inlineStr">
@@ -2999,24 +2951,37 @@
       </c>
       <c r="C69" s="25" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="D69" s="25" t="inlineStr">
         <is>
-          <t>Maghrib — surau Shibuya PARCO 5F</t>
-        </is>
-      </c>
-      <c r="E69" s="25" t="inlineStr">
-        <is>
-          <t>Maghrib 16:45</t>
-        </is>
-      </c>
-      <c r="F69" s="25" t="n"/>
-      <c r="G69" s="25" t="n"/>
-      <c r="H69" s="25" t="n"/>
-      <c r="I69" s="26" t="n"/>
-      <c r="J69" s="26" t="n"/>
+          <t>Lunch — Halal Wagyu Karemen King (Akihabara)</t>
+        </is>
+      </c>
+      <c r="E69" s="25" t="n"/>
+      <c r="F69" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G69" s="25" t="inlineStr">
+        <is>
+          <t>Buka 12:00-23:00</t>
+        </is>
+      </c>
+      <c r="H69" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I69" s="26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="J69" s="26">
+        <f>I69*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="27.75" customHeight="1" s="23">
       <c r="A70" s="25" t="inlineStr">
@@ -3031,37 +2996,20 @@
       </c>
       <c r="C70" s="25" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>Akihabara + dinner halal (Halal Wagyu Karemen King)</t>
+          <t>Gerak ke Shibuya (~30min)</t>
         </is>
       </c>
       <c r="E70" s="25" t="n"/>
-      <c r="F70" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
-      <c r="G70" s="25" t="inlineStr">
-        <is>
-          <t>Masjid Nusantara ~4min dari Karemen King</t>
-        </is>
-      </c>
-      <c r="H70" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I70" s="26" t="n">
-        <v>2200</v>
-      </c>
-      <c r="J70" s="26">
-        <f>I70*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="F70" s="25" t="n"/>
+      <c r="G70" s="25" t="n"/>
+      <c r="H70" s="25" t="n"/>
+      <c r="I70" s="26" t="n"/>
+      <c r="J70" s="26" t="n"/>
     </row>
     <row r="71" ht="27.75" customHeight="1" s="23">
       <c r="A71" s="25" t="inlineStr">
@@ -3076,17 +3024,17 @@
       </c>
       <c r="C71" s="25" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="D71" s="25" t="inlineStr">
         <is>
-          <t>Isyak (Masjid Nusantara, Akihabara)</t>
+          <t>Asar — surau Shibuya PARCO 5F</t>
         </is>
       </c>
       <c r="E71" s="25" t="inlineStr">
         <is>
-          <t>Isyak 18:05</t>
+          <t>Asar 14:20</t>
         </is>
       </c>
       <c r="F71" s="25" t="n"/>
@@ -3108,117 +3056,133 @@
       </c>
       <c r="C72" s="25" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D72" s="25" t="inlineStr">
         <is>
-          <t>Ambil bagasi dari coin locker, ke Busta Shinjuku</t>
+          <t>Shibuya Sky — slot 14:45 (OPTIONAL, boleh skip)</t>
         </is>
       </c>
       <c r="E72" s="25" t="n"/>
       <c r="F72" s="25" t="n"/>
-      <c r="G72" s="25" t="n"/>
-      <c r="H72" s="25" t="n"/>
-      <c r="I72" s="26" t="n"/>
-      <c r="J72" s="26" t="n"/>
+      <c r="G72" s="25" t="inlineStr">
+        <is>
+          <t>¥2,700 online (slot sebelum 15:00). Tiket untuk Ahad 10 Jan buka 27 Dis 00:00. Keluar sebelum Maghrib ~16:45</t>
+        </is>
+      </c>
+      <c r="H72" s="25" t="inlineStr">
+        <is>
+          <t>Attraction-Optional</t>
+        </is>
+      </c>
+      <c r="I72" s="26" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J72" s="26">
+        <f>I72*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="27.75" customHeight="1" s="23">
-      <c r="A73" s="31" t="inlineStr">
+      <c r="A73" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B73" s="31" t="inlineStr">
+      <c r="B73" s="25" t="inlineStr">
         <is>
           <t>10 Jan 2027</t>
         </is>
       </c>
-      <c r="C73" s="31" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D73" s="31" t="inlineStr">
-        <is>
-          <t>Bas overnight Tokyo (Busta Shinjuku) → Osaka (tidur atas bas)</t>
-        </is>
-      </c>
-      <c r="E73" s="31" t="n"/>
-      <c r="F73" s="31" t="n"/>
-      <c r="G73" s="31" t="inlineStr">
-        <is>
-          <t>Willer Express ~¥3,000-5,000, ~8-10j. Ahad cuti panjang — book awal</t>
-        </is>
-      </c>
-      <c r="H73" s="31" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I73" s="32" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J73" s="32">
-        <f>I73*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="C73" s="25" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib — surau Shibuya PARCO 5F</t>
+        </is>
+      </c>
+      <c r="E73" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib 16:45</t>
+        </is>
+      </c>
+      <c r="F73" s="25" t="n"/>
+      <c r="G73" s="25" t="n"/>
+      <c r="H73" s="25" t="n"/>
+      <c r="I73" s="26" t="n"/>
+      <c r="J73" s="26" t="n"/>
     </row>
     <row r="74" ht="27.75" customHeight="1" s="23">
-      <c r="A74" s="27" t="inlineStr">
-        <is>
-          <t>6
-(Isnin)</t>
-        </is>
-      </c>
-      <c r="B74" s="27" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C74" s="27" t="inlineStr">
-        <is>
-          <t>~05:38</t>
-        </is>
-      </c>
-      <c r="D74" s="27" t="inlineStr">
-        <is>
-          <t>Subuh (atas bas — anggar kiblat)</t>
-        </is>
-      </c>
-      <c r="E74" s="27" t="inlineStr">
-        <is>
-          <t>Subuh ~05:38</t>
-        </is>
-      </c>
-      <c r="F74" s="27" t="n"/>
-      <c r="G74" s="27" t="n"/>
-      <c r="H74" s="27" t="n"/>
-      <c r="I74" s="28" t="n"/>
-      <c r="J74" s="28" t="n"/>
+      <c r="A74" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B74" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C74" s="25" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="inlineStr">
+        <is>
+          <t>Dinner — halal Shibuya/Shinjuku</t>
+        </is>
+      </c>
+      <c r="E74" s="25" t="n"/>
+      <c r="F74" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G74" s="25" t="n"/>
+      <c r="H74" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I74" s="26" t="n">
+        <v>2200</v>
+      </c>
+      <c r="J74" s="26">
+        <f>I74*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="75" ht="27.75" customHeight="1" s="23">
       <c r="A75" s="25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>11 Jan 2027</t>
+          <t>10 Jan 2027</t>
         </is>
       </c>
       <c r="C75" s="25" t="inlineStr">
         <is>
-          <t>~07:30</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="D75" s="25" t="inlineStr">
         <is>
-          <t>Sampai Osaka (bas malam Willer, ~07:00-09:00) → terus balik guesthouse, mandi, tidur sekejap</t>
-        </is>
-      </c>
-      <c r="E75" s="25" t="n"/>
+          <t>Isyak</t>
+        </is>
+      </c>
+      <c r="E75" s="25" t="inlineStr">
+        <is>
+          <t>Isyak 18:05</t>
+        </is>
+      </c>
       <c r="F75" s="25" t="n"/>
       <c r="G75" s="25" t="n"/>
       <c r="H75" s="25" t="n"/>
@@ -3226,118 +3190,106 @@
       <c r="J75" s="26" t="n"/>
     </row>
     <row r="76" ht="27.75" customHeight="1" s="23">
-      <c r="A76" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B76" s="29" t="inlineStr">
+      <c r="A76" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B76" s="25" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C76" s="25" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="D76" s="25" t="inlineStr">
+        <is>
+          <t>Ambil bagasi dari coin locker, ke Busta Shinjuku</t>
+        </is>
+      </c>
+      <c r="E76" s="25" t="n"/>
+      <c r="F76" s="25" t="n"/>
+      <c r="G76" s="25" t="n"/>
+      <c r="H76" s="25" t="n"/>
+      <c r="I76" s="26" t="n"/>
+      <c r="J76" s="26" t="n"/>
+    </row>
+    <row r="77" ht="27.75" customHeight="1" s="23">
+      <c r="A77" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B77" s="31" t="inlineStr">
+        <is>
+          <t>10 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C77" s="31" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D77" s="31" t="inlineStr">
+        <is>
+          <t>Bas overnight Tokyo (Busta Shinjuku) → Osaka (tidur atas bas)</t>
+        </is>
+      </c>
+      <c r="E77" s="31" t="n"/>
+      <c r="F77" s="31" t="n"/>
+      <c r="G77" s="31" t="inlineStr">
+        <is>
+          <t>Willer Express ~¥3,000-5,000, ~8-10j. Ahad cuti panjang — book awal</t>
+        </is>
+      </c>
+      <c r="H77" s="31" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J77" s="32">
+        <f>I77*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" ht="27.75" customHeight="1" s="23">
+      <c r="A78" s="27" t="inlineStr">
+        <is>
+          <t>6
+(Isnin)</t>
+        </is>
+      </c>
+      <c r="B78" s="27" t="inlineStr">
         <is>
           <t>11 Jan 2027</t>
         </is>
       </c>
-      <c r="C76" s="29" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D76" s="29" t="inlineStr">
-        <is>
-          <t>Breakfast — masak kat guesthouse</t>
-        </is>
-      </c>
-      <c r="E76" s="29" t="n"/>
-      <c r="F76" s="29" t="inlineStr">
-        <is>
-          <t>Masak</t>
-        </is>
-      </c>
-      <c r="G76" s="29" t="n"/>
-      <c r="H76" s="29" t="inlineStr">
-        <is>
-          <t>Food-Masak</t>
-        </is>
-      </c>
-      <c r="I76" s="30" t="n">
-        <v>600</v>
-      </c>
-      <c r="J76" s="30">
-        <f>I76*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="27.75" customHeight="1" s="23">
-      <c r="A77" s="25" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B77" s="25" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C77" s="25" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D77" s="25" t="inlineStr">
-        <is>
-          <t>Gerak ke Kyoto: Midosuji Namba → Yodoyabashi, tukar Keihan → Kiyomizu-Gojo</t>
-        </is>
-      </c>
-      <c r="E77" s="25" t="n"/>
-      <c r="F77" s="25" t="n"/>
-      <c r="G77" s="25" t="inlineStr">
-        <is>
-          <t>¥240 + ¥430, ~1j15m. Isnin 11 Jan = CUTI UMUM Jepun (Seijin no Hi), Kyoto sesak</t>
-        </is>
-      </c>
-      <c r="H77" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I77" s="26" t="n">
-        <v>670</v>
-      </c>
-      <c r="J77" s="26">
-        <f>I77*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" ht="27.75" customHeight="1" s="23">
-      <c r="A78" s="25" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B78" s="25" t="inlineStr">
-        <is>
-          <t>11 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C78" s="25" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="D78" s="25" t="inlineStr">
-        <is>
-          <t>Zohor — ruang solat Shinjuku-tei Kiyomizu (restoran buka 12:00)</t>
-        </is>
-      </c>
-      <c r="E78" s="25" t="inlineStr">
-        <is>
-          <t>Zohor 12:00</t>
-        </is>
-      </c>
-      <c r="F78" s="25" t="n"/>
-      <c r="G78" s="25" t="n"/>
-      <c r="H78" s="25" t="n"/>
-      <c r="I78" s="26" t="n"/>
-      <c r="J78" s="26" t="n"/>
+      <c r="C78" s="27" t="inlineStr">
+        <is>
+          <t>~05:38</t>
+        </is>
+      </c>
+      <c r="D78" s="27" t="inlineStr">
+        <is>
+          <t>Subuh (atas bas — anggar kiblat)</t>
+        </is>
+      </c>
+      <c r="E78" s="27" t="inlineStr">
+        <is>
+          <t>Subuh ~05:38</t>
+        </is>
+      </c>
+      <c r="F78" s="27" t="n"/>
+      <c r="G78" s="27" t="n"/>
+      <c r="H78" s="27" t="n"/>
+      <c r="I78" s="28" t="n"/>
+      <c r="J78" s="28" t="n"/>
     </row>
     <row r="79" ht="27.75" customHeight="1" s="23">
       <c r="A79" s="25" t="inlineStr">
@@ -3352,75 +3304,58 @@
       </c>
       <c r="C79" s="25" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>~07:30</t>
         </is>
       </c>
       <c r="D79" s="25" t="inlineStr">
         <is>
-          <t>Lunch — HALAL WAGYU RAMEN SHINJUKU-TEI Kiyomizu (halal, ada ruang solat)</t>
+          <t>Sampai Osaka (bas malam Willer, ~07:00-09:00) → terus balik guesthouse, mandi, tidur sekejap</t>
         </is>
       </c>
       <c r="E79" s="25" t="n"/>
-      <c r="F79" s="25" t="inlineStr">
-        <is>
-          <t>Makan luar (halal)</t>
-        </is>
-      </c>
-      <c r="G79" s="25" t="inlineStr">
-        <is>
-          <t>148 Hoshinocho, dekat Ninenzaka. Chicken paitan ¥1,500-2,500; wagyu ramen ¥4,500. Backup: Halal Ramen Honolu Premier, Gion (buka 11:30)</t>
-        </is>
-      </c>
-      <c r="H79" s="25" t="inlineStr">
-        <is>
-          <t>Food-Luar</t>
-        </is>
-      </c>
-      <c r="I79" s="26" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J79" s="26">
-        <f>I79*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="F79" s="25" t="n"/>
+      <c r="G79" s="25" t="n"/>
+      <c r="H79" s="25" t="n"/>
+      <c r="I79" s="26" t="n"/>
+      <c r="J79" s="26" t="n"/>
     </row>
     <row r="80" ht="27.75" customHeight="1" s="23">
-      <c r="A80" s="25" t="inlineStr">
+      <c r="A80" s="29" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B80" s="25" t="inlineStr">
+      <c r="B80" s="29" t="inlineStr">
         <is>
           <t>11 Jan 2027</t>
         </is>
       </c>
-      <c r="C80" s="25" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="D80" s="25" t="inlineStr">
-        <is>
-          <t>Kiyomizu-dera (jalan naik Ninenzaka/Sannenzaka)</t>
-        </is>
-      </c>
-      <c r="E80" s="25" t="n"/>
-      <c r="F80" s="25" t="n"/>
-      <c r="G80" s="25" t="inlineStr">
-        <is>
-          <t>¥500, bayar TUNAI. Buka 06:00-18:00. Jalan dari stesen curam ~25min; teksi kongsi 6 orang pun murah</t>
-        </is>
-      </c>
-      <c r="H80" s="25" t="inlineStr">
-        <is>
-          <t>Attraction-Optional</t>
-        </is>
-      </c>
-      <c r="I80" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="J80" s="26">
+      <c r="C80" s="29" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>Breakfast — masak kat guesthouse</t>
+        </is>
+      </c>
+      <c r="E80" s="29" t="n"/>
+      <c r="F80" s="29" t="inlineStr">
+        <is>
+          <t>Masak</t>
+        </is>
+      </c>
+      <c r="G80" s="29" t="n"/>
+      <c r="H80" s="29" t="inlineStr">
+        <is>
+          <t>Food-Masak</t>
+        </is>
+      </c>
+      <c r="I80" s="30" t="n">
+        <v>600</v>
+      </c>
+      <c r="J80" s="30">
         <f>I80*'Budget Summary'!$B$2</f>
         <v/>
       </c>
@@ -3438,24 +3373,33 @@
       </c>
       <c r="C81" s="25" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D81" s="25" t="inlineStr">
         <is>
-          <t>Asar (kawasan Kiyomizu / surau restoran halal berdekatan)</t>
-        </is>
-      </c>
-      <c r="E81" s="25" t="inlineStr">
-        <is>
-          <t>Asar 14:35</t>
-        </is>
-      </c>
+          <t>Gerak ke Kyoto: Midosuji Namba → Yodoyabashi, tukar Keihan → Kiyomizu-Gojo</t>
+        </is>
+      </c>
+      <c r="E81" s="25" t="n"/>
       <c r="F81" s="25" t="n"/>
-      <c r="G81" s="25" t="n"/>
-      <c r="H81" s="25" t="n"/>
-      <c r="I81" s="26" t="n"/>
-      <c r="J81" s="26" t="n"/>
+      <c r="G81" s="25" t="inlineStr">
+        <is>
+          <t>¥240 + ¥430, ~1j15m. Isnin 11 Jan = CUTI UMUM Jepun (Seijin no Hi), Kyoto sesak</t>
+        </is>
+      </c>
+      <c r="H81" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I81" s="26" t="n">
+        <v>670</v>
+      </c>
+      <c r="J81" s="26">
+        <f>I81*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="82" ht="27.75" customHeight="1" s="23">
       <c r="A82" s="25" t="inlineStr">
@@ -3470,33 +3414,24 @@
       </c>
       <c r="C82" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D82" s="25" t="inlineStr">
         <is>
-          <t>Balik Osaka: Keihan Kiyomizu-Gojo → Yodoyabashi → Midosuji → Namba</t>
-        </is>
-      </c>
-      <c r="E82" s="25" t="n"/>
+          <t>Zohor — ruang solat Shinjuku-tei Kiyomizu (restoran buka 12:00)</t>
+        </is>
+      </c>
+      <c r="E82" s="25" t="inlineStr">
+        <is>
+          <t>Zohor 12:00</t>
+        </is>
+      </c>
       <c r="F82" s="25" t="n"/>
-      <c r="G82" s="25" t="inlineStr">
-        <is>
-          <t>¥430 + ¥240, ~1j15m. Sampai Namba ~16:45</t>
-        </is>
-      </c>
-      <c r="H82" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I82" s="26" t="n">
-        <v>670</v>
-      </c>
-      <c r="J82" s="26">
-        <f>I82*'Budget Summary'!$B$2</f>
-        <v/>
-      </c>
+      <c r="G82" s="25" t="n"/>
+      <c r="H82" s="25" t="n"/>
+      <c r="I82" s="26" t="n"/>
+      <c r="J82" s="26" t="n"/>
     </row>
     <row r="83" ht="27.75" customHeight="1" s="23">
       <c r="A83" s="25" t="inlineStr">
@@ -3511,62 +3446,75 @@
       </c>
       <c r="C83" s="25" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="D83" s="25" t="inlineStr">
         <is>
-          <t>Maghrib</t>
-        </is>
-      </c>
-      <c r="E83" s="25" t="inlineStr">
-        <is>
-          <t>Maghrib 17:00</t>
-        </is>
-      </c>
-      <c r="F83" s="25" t="n"/>
-      <c r="G83" s="25" t="n"/>
-      <c r="H83" s="25" t="n"/>
-      <c r="I83" s="26" t="n"/>
-      <c r="J83" s="26" t="n"/>
+          <t>Lunch — HALAL WAGYU RAMEN SHINJUKU-TEI Kiyomizu (halal, ada ruang solat)</t>
+        </is>
+      </c>
+      <c r="E83" s="25" t="n"/>
+      <c r="F83" s="25" t="inlineStr">
+        <is>
+          <t>Makan luar (halal)</t>
+        </is>
+      </c>
+      <c r="G83" s="25" t="inlineStr">
+        <is>
+          <t>148 Hoshinocho, dekat Ninenzaka. Chicken paitan ¥1,500-2,500; wagyu ramen ¥4,500. Backup: Halal Ramen Honolu Premier, Gion (buka 11:30)</t>
+        </is>
+      </c>
+      <c r="H83" s="25" t="inlineStr">
+        <is>
+          <t>Food-Luar</t>
+        </is>
+      </c>
+      <c r="I83" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J83" s="26">
+        <f>I83*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="84" ht="27.75" customHeight="1" s="23">
-      <c r="A84" s="29" t="inlineStr">
+      <c r="A84" s="25" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B84" s="29" t="inlineStr">
+      <c r="B84" s="25" t="inlineStr">
         <is>
           <t>11 Jan 2027</t>
         </is>
       </c>
-      <c r="C84" s="29" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="D84" s="29" t="inlineStr">
-        <is>
-          <t>Dinner — masak (habiskan baki bahan)</t>
-        </is>
-      </c>
-      <c r="E84" s="29" t="n"/>
-      <c r="F84" s="29" t="inlineStr">
-        <is>
-          <t>Masak</t>
-        </is>
-      </c>
-      <c r="G84" s="29" t="n"/>
-      <c r="H84" s="29" t="inlineStr">
-        <is>
-          <t>Food-Masak</t>
-        </is>
-      </c>
-      <c r="I84" s="30" t="n">
-        <v>700</v>
-      </c>
-      <c r="J84" s="30">
+      <c r="C84" s="25" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D84" s="25" t="inlineStr">
+        <is>
+          <t>Kiyomizu-dera (jalan naik Ninenzaka/Sannenzaka)</t>
+        </is>
+      </c>
+      <c r="E84" s="25" t="n"/>
+      <c r="F84" s="25" t="n"/>
+      <c r="G84" s="25" t="inlineStr">
+        <is>
+          <t>¥500, bayar TUNAI. Buka 06:00-18:00. Jalan dari stesen curam ~25min; teksi kongsi 6 orang pun murah</t>
+        </is>
+      </c>
+      <c r="H84" s="25" t="inlineStr">
+        <is>
+          <t>Attraction-Optional</t>
+        </is>
+      </c>
+      <c r="I84" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="J84" s="26">
         <f>I84*'Budget Summary'!$B$2</f>
         <v/>
       </c>
@@ -3584,17 +3532,17 @@
       </c>
       <c r="C85" s="25" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="D85" s="25" t="inlineStr">
         <is>
-          <t>Isyak</t>
+          <t>Asar (kawasan Kiyomizu / surau restoran halal berdekatan)</t>
         </is>
       </c>
       <c r="E85" s="25" t="inlineStr">
         <is>
-          <t>Isyak 18:20</t>
+          <t>Asar 14:35</t>
         </is>
       </c>
       <c r="F85" s="25" t="n"/>
@@ -3616,87 +3564,103 @@
       </c>
       <c r="C86" s="25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D86" s="25" t="inlineStr">
         <is>
-          <t>Kemas beg, tidur awal (flight awal esok!)</t>
+          <t>Balik Osaka: Keihan Kiyomizu-Gojo → Yodoyabashi → Midosuji → Namba</t>
         </is>
       </c>
       <c r="E86" s="25" t="n"/>
       <c r="F86" s="25" t="n"/>
-      <c r="G86" s="25" t="n"/>
-      <c r="H86" s="25" t="n"/>
-      <c r="I86" s="26" t="n"/>
-      <c r="J86" s="26" t="n"/>
+      <c r="G86" s="25" t="inlineStr">
+        <is>
+          <t>¥430 + ¥240, ~1j15m. Sampai Namba ~16:45</t>
+        </is>
+      </c>
+      <c r="H86" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I86" s="26" t="n">
+        <v>670</v>
+      </c>
+      <c r="J86" s="26">
+        <f>I86*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="87" ht="27.75" customHeight="1" s="23">
-      <c r="A87" s="27" t="inlineStr">
-        <is>
-          <t>7
-(Selasa)</t>
-        </is>
-      </c>
-      <c r="B87" s="27" t="inlineStr">
-        <is>
-          <t>12 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C87" s="27" t="inlineStr">
-        <is>
-          <t>~04:30</t>
-        </is>
-      </c>
-      <c r="D87" s="27" t="inlineStr">
-        <is>
-          <t>Bangun awal</t>
-        </is>
-      </c>
-      <c r="E87" s="27" t="n"/>
-      <c r="F87" s="27" t="n"/>
-      <c r="G87" s="27" t="n"/>
-      <c r="H87" s="27" t="n"/>
-      <c r="I87" s="28" t="n"/>
-      <c r="J87" s="28" t="n"/>
+      <c r="A87" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B87" s="25" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D87" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib</t>
+        </is>
+      </c>
+      <c r="E87" s="25" t="inlineStr">
+        <is>
+          <t>Maghrib 17:00</t>
+        </is>
+      </c>
+      <c r="F87" s="25" t="n"/>
+      <c r="G87" s="25" t="n"/>
+      <c r="H87" s="25" t="n"/>
+      <c r="I87" s="26" t="n"/>
+      <c r="J87" s="26" t="n"/>
     </row>
     <row r="88" ht="27.75" customHeight="1" s="23">
-      <c r="A88" s="25" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B88" s="25" t="inlineStr">
-        <is>
-          <t>12 Jan 2027</t>
-        </is>
-      </c>
-      <c r="C88" s="25" t="inlineStr">
-        <is>
-          <t>05:00</t>
-        </is>
-      </c>
-      <c r="D88" s="25" t="inlineStr">
-        <is>
-          <t>Nankai Airport Express Namba → KIX</t>
-        </is>
-      </c>
-      <c r="E88" s="25" t="n"/>
-      <c r="F88" s="25" t="n"/>
-      <c r="G88" s="25" t="inlineStr">
-        <is>
-          <t>¥970, ~45min</t>
-        </is>
-      </c>
-      <c r="H88" s="25" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="I88" s="26" t="n">
-        <v>970</v>
-      </c>
-      <c r="J88" s="26">
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>11 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D88" s="29" t="inlineStr">
+        <is>
+          <t>Dinner — masak (habiskan baki bahan)</t>
+        </is>
+      </c>
+      <c r="E88" s="29" t="n"/>
+      <c r="F88" s="29" t="inlineStr">
+        <is>
+          <t>Masak</t>
+        </is>
+      </c>
+      <c r="G88" s="29" t="n"/>
+      <c r="H88" s="29" t="inlineStr">
+        <is>
+          <t>Food-Masak</t>
+        </is>
+      </c>
+      <c r="I88" s="30" t="n">
+        <v>700</v>
+      </c>
+      <c r="J88" s="30">
         <f>I88*'Budget Summary'!$B$2</f>
         <v/>
       </c>
@@ -3704,27 +3668,27 @@
     <row r="89" ht="27.75" customHeight="1" s="23">
       <c r="A89" s="25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C89" s="25" t="inlineStr">
         <is>
-          <t>~05:38</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D89" s="25" t="inlineStr">
         <is>
-          <t>Subuh (kat guesthouse sblm gerak / atas train)</t>
+          <t>Isyak</t>
         </is>
       </c>
       <c r="E89" s="25" t="inlineStr">
         <is>
-          <t>Subuh ~05:38</t>
+          <t>Isyak 18:20</t>
         </is>
       </c>
       <c r="F89" s="25" t="n"/>
@@ -3736,62 +3700,59 @@
     <row r="90" ht="27.75" customHeight="1" s="23">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B90" s="25" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>11 Jan 2027</t>
         </is>
       </c>
       <c r="C90" s="25" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D90" s="25" t="inlineStr">
         <is>
-          <t>Sampai KIX — check-in, imigresen, security</t>
+          <t>Kemas beg, tidur awal (flight awal esok!)</t>
         </is>
       </c>
       <c r="E90" s="25" t="n"/>
       <c r="F90" s="25" t="n"/>
-      <c r="G90" s="25" t="inlineStr">
-        <is>
-          <t>Sampai ~2j sblm flight</t>
-        </is>
-      </c>
+      <c r="G90" s="25" t="n"/>
       <c r="H90" s="25" t="n"/>
       <c r="I90" s="26" t="n"/>
       <c r="J90" s="26" t="n"/>
     </row>
     <row r="91" ht="27.75" customHeight="1" s="23">
-      <c r="A91" s="25" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B91" s="25" t="inlineStr">
+      <c r="A91" s="27" t="inlineStr">
+        <is>
+          <t>7
+(Selasa)</t>
+        </is>
+      </c>
+      <c r="B91" s="27" t="inlineStr">
         <is>
           <t>12 Jan 2027</t>
         </is>
       </c>
-      <c r="C91" s="25" t="inlineStr">
-        <is>
-          <t>07:10</t>
-        </is>
-      </c>
-      <c r="D91" s="25" t="inlineStr">
-        <is>
-          <t>Boarding</t>
-        </is>
-      </c>
-      <c r="E91" s="25" t="n"/>
-      <c r="F91" s="25" t="n"/>
-      <c r="G91" s="25" t="n"/>
-      <c r="H91" s="25" t="n"/>
-      <c r="I91" s="26" t="n"/>
-      <c r="J91" s="26" t="n"/>
+      <c r="C91" s="27" t="inlineStr">
+        <is>
+          <t>~04:30</t>
+        </is>
+      </c>
+      <c r="D91" s="27" t="inlineStr">
+        <is>
+          <t>Bangun awal</t>
+        </is>
+      </c>
+      <c r="E91" s="27" t="n"/>
+      <c r="F91" s="27" t="n"/>
+      <c r="G91" s="27" t="n"/>
+      <c r="H91" s="27" t="n"/>
+      <c r="I91" s="28" t="n"/>
+      <c r="J91" s="28" t="n"/>
     </row>
     <row r="92" ht="27.75" customHeight="1" s="23">
       <c r="A92" s="25" t="inlineStr">
@@ -3806,20 +3767,153 @@
       </c>
       <c r="C92" s="25" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>05:00</t>
         </is>
       </c>
       <c r="D92" s="25" t="inlineStr">
         <is>
-          <t>Take off — balik Incheon</t>
+          <t>Nankai Airport Express Namba → KIX</t>
         </is>
       </c>
       <c r="E92" s="25" t="n"/>
       <c r="F92" s="25" t="n"/>
-      <c r="G92" s="25" t="n"/>
-      <c r="H92" s="25" t="n"/>
-      <c r="I92" s="26" t="n"/>
-      <c r="J92" s="26" t="n"/>
+      <c r="G92" s="25" t="inlineStr">
+        <is>
+          <t>¥970, ~45min</t>
+        </is>
+      </c>
+      <c r="H92" s="25" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="I92" s="26" t="n">
+        <v>970</v>
+      </c>
+      <c r="J92" s="26">
+        <f>I92*'Budget Summary'!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="27.75" customHeight="1" s="23">
+      <c r="A93" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B93" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C93" s="25" t="inlineStr">
+        <is>
+          <t>~05:38</t>
+        </is>
+      </c>
+      <c r="D93" s="25" t="inlineStr">
+        <is>
+          <t>Subuh (kat guesthouse sblm gerak / atas train)</t>
+        </is>
+      </c>
+      <c r="E93" s="25" t="inlineStr">
+        <is>
+          <t>Subuh ~05:38</t>
+        </is>
+      </c>
+      <c r="F93" s="25" t="n"/>
+      <c r="G93" s="25" t="n"/>
+      <c r="H93" s="25" t="n"/>
+      <c r="I93" s="26" t="n"/>
+      <c r="J93" s="26" t="n"/>
+    </row>
+    <row r="94" ht="27.75" customHeight="1" s="23">
+      <c r="A94" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B94" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C94" s="25" t="inlineStr">
+        <is>
+          <t>05:50</t>
+        </is>
+      </c>
+      <c r="D94" s="25" t="inlineStr">
+        <is>
+          <t>Sampai KIX — check-in, imigresen, security</t>
+        </is>
+      </c>
+      <c r="E94" s="25" t="n"/>
+      <c r="F94" s="25" t="n"/>
+      <c r="G94" s="25" t="inlineStr">
+        <is>
+          <t>Sampai ~2j sblm flight</t>
+        </is>
+      </c>
+      <c r="H94" s="25" t="n"/>
+      <c r="I94" s="26" t="n"/>
+      <c r="J94" s="26" t="n"/>
+    </row>
+    <row r="95" ht="27.75" customHeight="1" s="23">
+      <c r="A95" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B95" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C95" s="25" t="inlineStr">
+        <is>
+          <t>07:10</t>
+        </is>
+      </c>
+      <c r="D95" s="25" t="inlineStr">
+        <is>
+          <t>Boarding</t>
+        </is>
+      </c>
+      <c r="E95" s="25" t="n"/>
+      <c r="F95" s="25" t="n"/>
+      <c r="G95" s="25" t="n"/>
+      <c r="H95" s="25" t="n"/>
+      <c r="I95" s="26" t="n"/>
+      <c r="J95" s="26" t="n"/>
+    </row>
+    <row r="96" ht="27.75" customHeight="1" s="23">
+      <c r="A96" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B96" s="25" t="inlineStr">
+        <is>
+          <t>12 Jan 2027</t>
+        </is>
+      </c>
+      <c r="C96" s="25" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="D96" s="25" t="inlineStr">
+        <is>
+          <t>Take off — balik Incheon</t>
+        </is>
+      </c>
+      <c r="E96" s="25" t="n"/>
+      <c r="F96" s="25" t="n"/>
+      <c r="G96" s="25" t="n"/>
+      <c r="H96" s="25" t="n"/>
+      <c r="I96" s="26" t="n"/>
+      <c r="J96" s="26" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3920,16 +4014,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="23">
-      <c r="A8" s="37" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Apartment Tokyo — 9STAY Bunkyo Otsuka (2 malam, ₩249,969 ÷ 6)</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>41662</v>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Dah booking ✓ (non-refundable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Jumlah dah bayar</t>
         </is>
       </c>
-      <c r="B8" s="38">
-        <f>SUM(B6:B7)</f>
-        <v/>
-      </c>
-      <c r="C8" s="37" t="n"/>
+      <c r="B9" s="38">
+        <f>SUM(B6:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="37" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="23">
       <c r="A10" s="33" t="inlineStr">
@@ -3967,7 +4076,7 @@
         </is>
       </c>
       <c r="B12" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E12,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E12,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C12" s="26">
@@ -3991,7 +4100,7 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E13,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E13,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C13" s="26">
@@ -4011,11 +4120,11 @@
     <row r="14" ht="15" customHeight="1" s="23">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>Penginapan tambahan (manga cafe Tokyo x1; malam Sabtu tidur dalam kereta)</t>
+          <t>Penginapan tambahan (Tokyo dah bayar — lihat atas)</t>
         </is>
       </c>
       <c r="B14" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E14,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E14,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C14" s="26">
@@ -4039,7 +4148,7 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E15,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E15,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C15" s="26">
@@ -4063,7 +4172,7 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E16,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E16,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C16" s="26">
@@ -4083,11 +4192,11 @@
     <row r="17" ht="15" customHeight="1" s="23">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>Makanan — bekal dibawa</t>
+          <t>Makanan — bekal/snek</t>
         </is>
       </c>
       <c r="B17" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E17,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E17,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C17" s="26">
@@ -4111,7 +4220,7 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>SUMIF(Itinerary!$H$2:$H$92,E18,Itinerary!$I$2:$I$92)</f>
+        <f>SUMIF(Itinerary!$H$2:$H$96,E18,Itinerary!$I$2:$I$96)</f>
         <v/>
       </c>
       <c r="C18" s="26">
@@ -4172,7 +4281,7 @@
         </is>
       </c>
       <c r="C23" s="39">
-        <f>B8+C19+C21</f>
+        <f>B9+C19+C21</f>
         <v/>
       </c>
     </row>
@@ -4190,7 +4299,7 @@
     <row r="26" ht="30" customHeight="1" s="23">
       <c r="A26" s="40" t="inlineStr">
         <is>
-          <t>Nota: Food-Bekal = snek malam + sarapan dalam kereta (Hari 4). Kereta sewa = anggaran Toyota W2 + tayar salji + insurans, SEMAK harga sebenar masa booking. Kos masak = anggaran groceries sahaja.</t>
+          <t>Nota: Kereta sewa = anggaran Toyota W2 + tayar salji + insurans, SEMAK harga sebenar masa booking. Parking semalaman Tokyo (Sab) ~¥2-3k — apartment takde parking. Kos masak = anggaran groceries sahaja.</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4462,7 @@
     <row r="13" ht="45" customHeight="1" s="23">
       <c r="A13" s="43" t="inlineStr">
         <is>
-          <t>PENTING — Hari 3 &amp; 6: Subuh jatuh time atas bas overnight. Sedia air sembahyang/tayammum kering, guna qiblat app, dan boleh jamak/qada bila sampai kalau betul-betul tak boleh solat atas bas. Hari 5: Subuh di tepi tasik Kawaguchiko (bawa sejadah).</t>
+          <t>PENTING — Hari 3 &amp; 6: Subuh jatuh time atas bas overnight. Sedia air sembahyang/tayammum kering, guna qiblat app, dan boleh jamak/qada bila sampai kalau betul-betul tak boleh solat atas bas.</t>
         </is>
       </c>
     </row>

</xml_diff>